<commit_message>
Populate Volume / Specs & Prices / Remarks from full email bodies
Re-read the full body of every inbound product inquiry (~93 companies)
and extract Product Volume (col J), Product Specs & Prices (col L) and
Any Special Remarks (col N) - quantities/MOQ, technical specs, prices,
Incoterms, destination ports, certifications, payment terms and
deadlines. Trade-show / introduction contacts left blank.

Fill rate: Volume 47, Specs 86, Remarks 93 of 130 rows.
</commit_message>
<xml_diff>
--- a/Generic_Requests_filled.xlsx
+++ b/Generic_Requests_filled.xlsx
@@ -972,7 +972,7 @@
       <c r="N5" s="34" t="n"/>
       <c r="O5" s="35" t="n"/>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="46" customHeight="1">
       <c r="A6" s="36" t="n">
         <v>2</v>
       </c>
@@ -1008,14 +1008,26 @@
           <t>Bulk freeze-dried fruits</t>
         </is>
       </c>
-      <c r="J6" s="36" t="inlineStr"/>
+      <c r="J6" s="36" t="inlineStr">
+        <is>
+          <t>Tiered per SKU: 100-250 kg trial / 500-1,000 kg / 1,500-2,500 kg / 8,000+ kg full container</t>
+        </is>
+      </c>
       <c r="K6" s="38" t="n"/>
-      <c r="L6" s="36" t="inlineStr"/>
+      <c r="L6" s="36" t="inlineStr">
+        <is>
+          <t>Bulk FD fruits, all varieties (berries, tropical, stone, dates, exotic), whole &amp; sliced; moisture &lt;5%; bulk aluminium-foil laminate w/ nitrogen flush, OEM/retail-ready option</t>
+        </is>
+      </c>
       <c r="M6" s="38" t="n"/>
-      <c r="N6" s="36" t="inlineStr"/>
+      <c r="N6" s="36" t="inlineStr">
+        <is>
+          <t>FOB &amp; CIF Jeddah pricing; SFDA compliance; certs ISO22000/HACCP/FSSC22000, Halal, CoA, heavy-metals, pesticide &amp; micro reports; terms 30% deposit/70% vs B/L copy; M +966 547330506</t>
+        </is>
+      </c>
       <c r="O6" s="38" t="n"/>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="46" customHeight="1">
       <c r="A7" s="36" t="n">
         <v>3</v>
       </c>
@@ -1051,14 +1063,26 @@
           <t>Freeze-dried fruits</t>
         </is>
       </c>
-      <c r="J7" s="36" t="inlineStr"/>
+      <c r="J7" s="36" t="inlineStr">
+        <is>
+          <t>MOQ requested (not stated)</t>
+        </is>
+      </c>
       <c r="K7" s="38" t="n"/>
-      <c r="L7" s="36" t="inlineStr"/>
+      <c r="L7" s="36" t="inlineStr">
+        <is>
+          <t>FD strawberry (whole/pieces/slices/powder), blueberry, raspberry, cherry, black/red currant, pineapple, fig, peach, dragon fruit, kiwi, peas, corn; EU-compliant</t>
+        </is>
+      </c>
       <c r="M7" s="38" t="n"/>
-      <c r="N7" s="36" t="inlineStr"/>
+      <c r="N7" s="36" t="inlineStr">
+        <is>
+          <t>Wants catalogue + wholesale price list, MOQ, packaging options; long-term; Mob +370 687 32276</t>
+        </is>
+      </c>
       <c r="O7" s="38" t="n"/>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="46" customHeight="1">
       <c r="A8" s="36" t="n">
         <v>4</v>
       </c>
@@ -1096,12 +1120,20 @@
       </c>
       <c r="J8" s="36" t="inlineStr"/>
       <c r="K8" s="38" t="n"/>
-      <c r="L8" s="36" t="inlineStr"/>
+      <c r="L8" s="36" t="inlineStr">
+        <is>
+          <t>Orange &amp; lemon juice concentrate, Brix 60-65%</t>
+        </is>
+      </c>
       <c r="M8" s="38" t="n"/>
-      <c r="N8" s="36" t="inlineStr"/>
+      <c r="N8" s="36" t="inlineStr">
+        <is>
+          <t>Best offer requested; Al Safwa Group; tel 01020958645; al-safwagroup.com</t>
+        </is>
+      </c>
       <c r="O8" s="38" t="n"/>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="46" customHeight="1">
       <c r="A9" s="36" t="n">
         <v>5</v>
       </c>
@@ -1144,7 +1176,7 @@
       <c r="N9" s="36" t="inlineStr"/>
       <c r="O9" s="38" t="n"/>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="46" customHeight="1">
       <c r="A10" s="36" t="n">
         <v>6</v>
       </c>
@@ -1168,14 +1200,26 @@
           <t>Orange juice concentrate (RFQ)</t>
         </is>
       </c>
-      <c r="J10" s="36" t="inlineStr"/>
+      <c r="J10" s="36" t="inlineStr">
+        <is>
+          <t>25 MT</t>
+        </is>
+      </c>
       <c r="K10" s="38" t="n"/>
-      <c r="L10" s="36" t="inlineStr"/>
+      <c r="L10" s="36" t="inlineStr">
+        <is>
+          <t>FCOJ Brix 65 +/-1, acid/sugar ratio 12-15, pulp &lt;6%, high aroma &amp; cloud stability, Valencia oranges; 200-250 L steel drums w/ aseptic liner</t>
+        </is>
+      </c>
       <c r="M10" s="38" t="n"/>
-      <c r="N10" s="36" t="inlineStr"/>
+      <c r="N10" s="36" t="inlineStr">
+        <is>
+          <t>CIF Aden Port (Yemen); SGF + ISO22000/HACCP; L/C at sight; offer valid 15 days; deadline 15 May 2026; pre-shipment sample; +967 775289989</t>
+        </is>
+      </c>
       <c r="O10" s="38" t="n"/>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="46" customHeight="1">
       <c r="A11" s="36" t="n">
         <v>7</v>
       </c>
@@ -1211,14 +1255,26 @@
           <t>NFC juices (samples + quotation)</t>
         </is>
       </c>
-      <c r="J11" s="36" t="inlineStr"/>
+      <c r="J11" s="36" t="inlineStr">
+        <is>
+          <t>40 ft container (initial/annual)</t>
+        </is>
+      </c>
       <c r="K11" s="38" t="n"/>
-      <c r="L11" s="36" t="inlineStr"/>
+      <c r="L11" s="36" t="inlineStr">
+        <is>
+          <t>NFC juices in ready-to-sell 495 ml bottles / Tetra / aluminium cans, all flavours; samples for R&amp;D/private label</t>
+        </is>
+      </c>
       <c r="M11" s="38" t="n"/>
-      <c r="N11" s="36" t="inlineStr"/>
+      <c r="N11" s="36" t="inlineStr">
+        <is>
+          <t>FOB Alexandria; destination Port of Los Angeles; FDA compliance; +1 626 230 3697</t>
+        </is>
+      </c>
       <c r="O11" s="38" t="n"/>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="46" customHeight="1">
       <c r="A12" s="36" t="n">
         <v>8</v>
       </c>
@@ -1246,14 +1302,26 @@
           <t>Frozen strawberries, mango, puree</t>
         </is>
       </c>
-      <c r="J12" s="36" t="inlineStr"/>
+      <c r="J12" s="36" t="inlineStr">
+        <is>
+          <t>Open to volume commitment after offer (RFQ, FOB $/MT)</t>
+        </is>
+      </c>
       <c r="K12" s="38" t="n"/>
-      <c r="L12" s="36" t="inlineStr"/>
+      <c r="L12" s="36" t="inlineStr">
+        <is>
+          <t>IQF strawberries 1 kg/pack (Fortuna/Festival/Sensation, Grade A/B/BC, calibrated 15-25 &amp; 25-35); frozen mango slices/cubes (Zebdya/Kent) 1 kg; mango puree 1 kg; strawberry puree 1 kg</t>
+        </is>
+      </c>
       <c r="M12" s="38" t="n"/>
-      <c r="N12" s="36" t="inlineStr"/>
+      <c r="N12" s="36" t="inlineStr">
+        <is>
+          <t>FOB price/MT; certs ISO22000/GLOBALG.A.P./HACCP/Halal/BRC; COA &amp; MRLs; Italian shareholding; plans New Cairo office visit; +216 53531335</t>
+        </is>
+      </c>
       <c r="O12" s="38" t="n"/>
     </row>
-    <row r="13" ht="30" customHeight="1">
+    <row r="13" ht="46" customHeight="1">
       <c r="A13" s="36" t="n">
         <v>9</v>
       </c>
@@ -1287,12 +1355,20 @@
       </c>
       <c r="J13" s="36" t="inlineStr"/>
       <c r="K13" s="38" t="n"/>
-      <c r="L13" s="36" t="inlineStr"/>
+      <c r="L13" s="36" t="inlineStr">
+        <is>
+          <t>Supplier-side offer (not a buyer RFQ): Non-Dairy Creamer/fat-filled powder; Fruit &amp; Vegetable powders (mango, banana, beetroot, spinach); natural extracts &amp; colors; coconut/dairy ingredients; maltodextrin</t>
+        </is>
+      </c>
       <c r="M13" s="38" t="n"/>
-      <c r="N13" s="36" t="inlineStr"/>
+      <c r="N13" s="36" t="inlineStr">
+        <is>
+          <t>Met at Gulfood Dubai 2026; product catalogue attached; offers samples &amp; custom formulations; asks for MAFI's requirements; from Harshit Shukla, Venkatesh, India</t>
+        </is>
+      </c>
       <c r="O13" s="38" t="n"/>
     </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="14" ht="46" customHeight="1">
       <c r="A14" s="36" t="n">
         <v>10</v>
       </c>
@@ -1324,14 +1400,26 @@
           <t>Freeze-dried strawberries (15-25mm, 5 tons CIF Mersin)</t>
         </is>
       </c>
-      <c r="J14" s="36" t="inlineStr"/>
+      <c r="J14" s="36" t="inlineStr">
+        <is>
+          <t>5 tons</t>
+        </is>
+      </c>
       <c r="K14" s="38" t="n"/>
-      <c r="L14" s="36" t="inlineStr"/>
+      <c r="L14" s="36" t="inlineStr">
+        <is>
+          <t>FD strawberries, 15-25 mm festival calibrated</t>
+        </is>
+      </c>
       <c r="M14" s="38" t="n"/>
-      <c r="N14" s="36" t="inlineStr"/>
+      <c r="N14" s="36" t="inlineStr">
+        <is>
+          <t>CIF Mersin; also exploring IQF (Gulfood 2026 follow-up) &amp; market availability; M +90 542 761 5459</t>
+        </is>
+      </c>
       <c r="O14" s="38" t="n"/>
     </row>
-    <row r="15" ht="30" customHeight="1">
+    <row r="15" ht="46" customHeight="1">
       <c r="A15" s="36" t="n">
         <v>11</v>
       </c>
@@ -1363,14 +1451,26 @@
           <t>Fruit juice concentrates &amp; tomato paste</t>
         </is>
       </c>
-      <c r="J15" s="36" t="inlineStr"/>
+      <c r="J15" s="36" t="inlineStr">
+        <is>
+          <t>20ft container = 86 drums x 270 kg</t>
+        </is>
+      </c>
       <c r="K15" s="38" t="n"/>
-      <c r="L15" s="36" t="inlineStr"/>
+      <c r="L15" s="36" t="inlineStr">
+        <is>
+          <t>Supplier-side offer (not a buyer RFQ): pomegranate, apple, sour cherry, date juice concentrates &amp; tomato paste; aseptic bags in drums</t>
+        </is>
+      </c>
       <c r="M15" s="38" t="n"/>
-      <c r="N15" s="36" t="inlineStr"/>
+      <c r="N15" s="36" t="inlineStr">
+        <is>
+          <t>CFR Alexandria/Damietta; ETD 7-10 days after order, ETA Egypt ~32-35 days; met Mr. Amr Medany at Gulfood; Hojat Abdolahi, Dubai, +971569736002</t>
+        </is>
+      </c>
       <c r="O15" s="38" t="n"/>
     </row>
-    <row r="16" ht="30" customHeight="1">
+    <row r="16" ht="46" customHeight="1">
       <c r="A16" s="36" t="n">
         <v>12</v>
       </c>
@@ -1406,14 +1506,26 @@
           <t>Wet strawberry/blackberry/kiwi pomace &amp; seeds (20-200 tons)</t>
         </is>
       </c>
-      <c r="J16" s="36" t="inlineStr"/>
+      <c r="J16" s="36" t="inlineStr">
+        <is>
+          <t>20 to 200 tons of each by-product</t>
+        </is>
+      </c>
       <c r="K16" s="38" t="n"/>
-      <c r="L16" s="36" t="inlineStr"/>
+      <c r="L16" s="36" t="inlineStr">
+        <is>
+          <t>Wet strawberry pomace/seeds (from puree production), wet blackberry pomace, wet kiwi pomace (from puree/NFC/concentrate); packed frozen in used drums</t>
+        </is>
+      </c>
       <c r="M16" s="38" t="n"/>
-      <c r="N16" s="36" t="inlineStr"/>
+      <c r="N16" s="36" t="inlineStr">
+        <is>
+          <t>Requests price offer, available qty, photos, lead time; buying strawberry now as season started; upcycling/circular economy; Daniel Polak, GreenField Poland, WhatsApp +48 510 410 180</t>
+        </is>
+      </c>
       <c r="O16" s="38" t="n"/>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="46" customHeight="1">
       <c r="A17" s="36" t="n">
         <v>13</v>
       </c>
@@ -1453,14 +1565,26 @@
           <t>Conventional FD fruits</t>
         </is>
       </c>
-      <c r="J17" s="36" t="inlineStr"/>
+      <c r="J17" s="36" t="inlineStr">
+        <is>
+          <t>~50 tons/year; orders by full 40ft FCL container</t>
+        </is>
+      </c>
       <c r="K17" s="38" t="n"/>
-      <c r="L17" s="36" t="inlineStr"/>
+      <c r="L17" s="36" t="inlineStr">
+        <is>
+          <t>Conventional FD strawberry slices 5-7mm (also dices 5-10mm or mix); max 5-7% moisture, max 5% dust; no sugar/additives, 100% fruit, no pesticide residue; requests current price offer</t>
+        </is>
+      </c>
       <c r="M17" s="38" t="n"/>
-      <c r="N17" s="36" t="inlineStr"/>
+      <c r="N17" s="36" t="inlineStr">
+        <is>
+          <t>Kosher certified, gluten up to 10ppm; DAP Czech Republic, Hrdly 412 01; long-term cooperation; Jakub Fric, Emco, +420 771 257 818</t>
+        </is>
+      </c>
       <c r="O17" s="38" t="n"/>
     </row>
-    <row r="18" ht="30" customHeight="1">
+    <row r="18" ht="46" customHeight="1">
       <c r="A18" s="36" t="n">
         <v>14</v>
       </c>
@@ -1494,12 +1618,20 @@
       </c>
       <c r="J18" s="36" t="inlineStr"/>
       <c r="K18" s="38" t="n"/>
-      <c r="L18" s="36" t="inlineStr"/>
+      <c r="L18" s="36" t="inlineStr">
+        <is>
+          <t>Freeze-dried whole strawberries; requests product catalog and pricing</t>
+        </is>
+      </c>
       <c r="M18" s="38" t="n"/>
-      <c r="N18" s="36" t="inlineStr"/>
+      <c r="N18" s="36" t="inlineStr">
+        <is>
+          <t>EU food law compliance and delivery details requested; Pelian Lab Greece (healthy snacking); Nasos Drakopoulos</t>
+        </is>
+      </c>
       <c r="O18" s="38" t="n"/>
     </row>
-    <row r="19" ht="30" customHeight="1">
+    <row r="19" ht="46" customHeight="1">
       <c r="A19" s="36" t="n">
         <v>15</v>
       </c>
@@ -1542,7 +1674,7 @@
       <c r="N19" s="36" t="inlineStr"/>
       <c r="O19" s="38" t="n"/>
     </row>
-    <row r="20" ht="30" customHeight="1">
+    <row r="20" ht="46" customHeight="1">
       <c r="A20" s="36" t="n">
         <v>16</v>
       </c>
@@ -1580,12 +1712,20 @@
       </c>
       <c r="J20" s="36" t="inlineStr"/>
       <c r="K20" s="38" t="n"/>
-      <c r="L20" s="36" t="inlineStr"/>
+      <c r="L20" s="36" t="inlineStr">
+        <is>
+          <t>Freeze-dried strawberries, blueberries, raspberries, cherries; particularly interested in whole raspberries; requests product range details</t>
+        </is>
+      </c>
       <c r="M20" s="38" t="n"/>
-      <c r="N20" s="36" t="inlineStr"/>
+      <c r="N20" s="36" t="inlineStr">
+        <is>
+          <t>Met at SIAL Paris 2024; has several customers interested; LitSupply (food raw materials supplier); Justinas Grazelis</t>
+        </is>
+      </c>
       <c r="O20" s="38" t="n"/>
     </row>
-    <row r="21" ht="30" customHeight="1">
+    <row r="21" ht="46" customHeight="1">
       <c r="A21" s="36" t="n">
         <v>17</v>
       </c>
@@ -1628,7 +1768,7 @@
       <c r="N21" s="36" t="inlineStr"/>
       <c r="O21" s="38" t="n"/>
     </row>
-    <row r="22" ht="30" customHeight="1">
+    <row r="22" ht="46" customHeight="1">
       <c r="A22" s="36" t="n">
         <v>18</v>
       </c>
@@ -1660,14 +1800,26 @@
           <t>Freeze-dried sliced strawberries (100-500kg)</t>
         </is>
       </c>
-      <c r="J22" s="36" t="inlineStr"/>
+      <c r="J22" s="36" t="inlineStr">
+        <is>
+          <t>100-500 kg</t>
+        </is>
+      </c>
       <c r="K22" s="38" t="n"/>
-      <c r="L22" s="36" t="inlineStr"/>
+      <c r="L22" s="36" t="inlineStr">
+        <is>
+          <t>Freeze-dried sliced strawberries, in bulk cartons; requests quote and a sample before buying</t>
+        </is>
+      </c>
       <c r="M22" s="38" t="n"/>
-      <c r="N22" s="36" t="inlineStr"/>
+      <c r="N22" s="36" t="inlineStr">
+        <is>
+          <t>Ship to Texas, likely Port of Houston; samples to CTD Sports, 5784 Sapp Road, Conroe, TX 77304, USA; Peter</t>
+        </is>
+      </c>
       <c r="O22" s="38" t="n"/>
     </row>
-    <row r="23" ht="30" customHeight="1">
+    <row r="23" ht="46" customHeight="1">
       <c r="A23" s="36" t="n">
         <v>19</v>
       </c>
@@ -1703,14 +1855,26 @@
           <t>Freeze-dried fruits / frozen mango</t>
         </is>
       </c>
-      <c r="J23" s="36" t="inlineStr"/>
+      <c r="J23" s="36" t="inlineStr">
+        <is>
+          <t>100 kg of each fruit ideally to start</t>
+        </is>
+      </c>
       <c r="K23" s="38" t="n"/>
-      <c r="L23" s="36" t="inlineStr"/>
+      <c r="L23" s="36" t="inlineStr">
+        <is>
+          <t>Freeze-dried fruits: strawberries, figs, orange, raspberry, blueberry, mulberry, pineapple, lemon; private labeling; requests prices</t>
+        </is>
+      </c>
       <c r="M23" s="38" t="n"/>
-      <c r="N23" s="36" t="inlineStr"/>
+      <c r="N23" s="36" t="inlineStr">
+        <is>
+          <t>Private label inquiry; prefers WhatsApp; Patrick, Sales Manager, Ginju, +1 (514) 299-1111, www.ginju.ca</t>
+        </is>
+      </c>
       <c r="O23" s="38" t="n"/>
     </row>
-    <row r="24" ht="30" customHeight="1">
+    <row r="24" ht="46" customHeight="1">
       <c r="A24" s="36" t="n">
         <v>20</v>
       </c>
@@ -1753,7 +1917,7 @@
       <c r="N24" s="36" t="inlineStr"/>
       <c r="O24" s="38" t="n"/>
     </row>
-    <row r="25" ht="30" customHeight="1">
+    <row r="25" ht="46" customHeight="1">
       <c r="A25" s="36" t="n">
         <v>21</v>
       </c>
@@ -1796,7 +1960,7 @@
       <c r="N25" s="36" t="inlineStr"/>
       <c r="O25" s="38" t="n"/>
     </row>
-    <row r="26" ht="30" customHeight="1">
+    <row r="26" ht="46" customHeight="1">
       <c r="A26" s="36" t="n">
         <v>22</v>
       </c>
@@ -1831,7 +1995,7 @@
       <c r="N26" s="36" t="inlineStr"/>
       <c r="O26" s="38" t="n"/>
     </row>
-    <row r="27" ht="30" customHeight="1">
+    <row r="27" ht="46" customHeight="1">
       <c r="A27" s="36" t="n">
         <v>23</v>
       </c>
@@ -1874,7 +2038,7 @@
       <c r="N27" s="36" t="inlineStr"/>
       <c r="O27" s="38" t="n"/>
     </row>
-    <row r="28" ht="30" customHeight="1">
+    <row r="28" ht="46" customHeight="1">
       <c r="A28" s="39" t="n">
         <v>24</v>
       </c>
@@ -1914,7 +2078,7 @@
       <c r="L28" s="39" t="inlineStr"/>
       <c r="N28" s="39" t="inlineStr"/>
     </row>
-    <row r="29" ht="30" customHeight="1">
+    <row r="29" ht="46" customHeight="1">
       <c r="A29" s="39" t="n">
         <v>25</v>
       </c>
@@ -1954,7 +2118,7 @@
       <c r="L29" s="39" t="inlineStr"/>
       <c r="N29" s="39" t="inlineStr"/>
     </row>
-    <row r="30" ht="30" customHeight="1">
+    <row r="30" ht="46" customHeight="1">
       <c r="A30" s="39" t="n">
         <v>26</v>
       </c>
@@ -1990,7 +2154,7 @@
       <c r="L30" s="39" t="inlineStr"/>
       <c r="N30" s="39" t="inlineStr"/>
     </row>
-    <row r="31" ht="30" customHeight="1">
+    <row r="31" ht="46" customHeight="1">
       <c r="A31" s="39" t="n">
         <v>27</v>
       </c>
@@ -2030,7 +2194,7 @@
       <c r="L31" s="39" t="inlineStr"/>
       <c r="N31" s="39" t="inlineStr"/>
     </row>
-    <row r="32" ht="30" customHeight="1">
+    <row r="32" ht="46" customHeight="1">
       <c r="A32" s="39" t="n">
         <v>28</v>
       </c>
@@ -2063,10 +2227,18 @@
         </is>
       </c>
       <c r="J32" s="39" t="inlineStr"/>
-      <c r="L32" s="39" t="inlineStr"/>
-      <c r="N32" s="39" t="inlineStr"/>
-    </row>
-    <row r="33" ht="30" customHeight="1">
+      <c r="L32" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried strawberry slices and freeze-dried raspberries; requests product catalog, price list and MOQs</t>
+        </is>
+      </c>
+      <c r="N32" s="39" t="inlineStr">
+        <is>
+          <t>Terms of cooperation requested; Polish company; Kamil Krzywonos, CEO, BILOW sp. z o.o., Rzeszow, +48 791 523 861</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="46" customHeight="1">
       <c r="A33" s="39" t="n">
         <v>29</v>
       </c>
@@ -2102,7 +2274,7 @@
       <c r="L33" s="39" t="inlineStr"/>
       <c r="N33" s="39" t="inlineStr"/>
     </row>
-    <row r="34" ht="30" customHeight="1">
+    <row r="34" ht="46" customHeight="1">
       <c r="A34" s="39" t="n">
         <v>30</v>
       </c>
@@ -2138,7 +2310,7 @@
       <c r="L34" s="39" t="inlineStr"/>
       <c r="N34" s="39" t="inlineStr"/>
     </row>
-    <row r="35" ht="30" customHeight="1">
+    <row r="35" ht="46" customHeight="1">
       <c r="A35" s="39" t="n">
         <v>31</v>
       </c>
@@ -2174,7 +2346,7 @@
       <c r="L35" s="39" t="inlineStr"/>
       <c r="N35" s="39" t="inlineStr"/>
     </row>
-    <row r="36" ht="30" customHeight="1">
+    <row r="36" ht="46" customHeight="1">
       <c r="A36" s="39" t="n">
         <v>32</v>
       </c>
@@ -2207,10 +2379,18 @@
         </is>
       </c>
       <c r="J36" s="39" t="inlineStr"/>
-      <c r="L36" s="39" t="inlineStr"/>
-      <c r="N36" s="39" t="inlineStr"/>
-    </row>
-    <row r="37" ht="30" customHeight="1">
+      <c r="L36" s="39" t="inlineStr">
+        <is>
+          <t>FC Orange Juice (66 Brix) and NFC orange juice; also other FC/NFC fruit juices with supply-chain advantages; requests quotation, MOQ, product info</t>
+        </is>
+      </c>
+      <c r="N36" s="39" t="inlineStr">
+        <is>
+          <t>FOB/CIF Main Chinese Ports; requests delivery time and payment terms; Alex Gao, Leyuan Health Technology, Hangzhou China; company intro PDF attached</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="46" customHeight="1">
       <c r="A37" s="39" t="n">
         <v>33</v>
       </c>
@@ -2246,7 +2426,7 @@
       <c r="L37" s="39" t="inlineStr"/>
       <c r="N37" s="39" t="inlineStr"/>
     </row>
-    <row r="38" ht="30" customHeight="1">
+    <row r="38" ht="46" customHeight="1">
       <c r="A38" s="39" t="n">
         <v>34</v>
       </c>
@@ -2274,11 +2454,23 @@
           <t>FD strawberries (slices, ~3 tonnes/yr)</t>
         </is>
       </c>
-      <c r="J38" s="39" t="inlineStr"/>
-      <c r="L38" s="39" t="inlineStr"/>
-      <c r="N38" s="39" t="inlineStr"/>
-    </row>
-    <row r="39" ht="30" customHeight="1">
+      <c r="J38" s="39" t="inlineStr">
+        <is>
+          <t>~3 tonnes per annum (sliced strawberries)</t>
+        </is>
+      </c>
+      <c r="L38" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried fruit; sliced strawberries; asks whether other fruits beyond strawberries are freeze-dried; requests price</t>
+        </is>
+      </c>
+      <c r="N38" s="39" t="inlineStr">
+        <is>
+          <t>Czech Republic food importer/distributor to ~400 stores; wants to start importing freeze-dried fruit; received brochure; Jaroslav</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="46" customHeight="1">
       <c r="A39" s="39" t="n">
         <v>35</v>
       </c>
@@ -2315,10 +2507,18 @@
         </is>
       </c>
       <c r="J39" s="39" t="inlineStr"/>
-      <c r="L39" s="39" t="inlineStr"/>
-      <c r="N39" s="39" t="inlineStr"/>
-    </row>
-    <row r="40" ht="30" customHeight="1">
+      <c r="L39" s="39" t="inlineStr">
+        <is>
+          <t>Private label/OEM dried strawberries &amp; bananas and fruit purees; requests MOQs, pricing structure (tiered + setup fees), packaging/custom branding capabilities</t>
+        </is>
+      </c>
+      <c r="N39" s="39" t="inlineStr">
+        <is>
+          <t>Lead times &amp; export compliance certs (ISO, HACCP, FDA, BRC) for EU &amp; Gulf/GCC markets; two-phase local-then-export rollout; Mohamed Fathy Helal, Alfa Trans, Cairo, +20227515755 / +201005622232; requests intro call</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="46" customHeight="1">
       <c r="A40" s="39" t="n">
         <v>36</v>
       </c>
@@ -2347,10 +2547,18 @@
         </is>
       </c>
       <c r="J40" s="39" t="inlineStr"/>
-      <c r="L40" s="39" t="inlineStr"/>
-      <c r="N40" s="39" t="inlineStr"/>
-    </row>
-    <row r="41" ht="30" customHeight="1">
+      <c r="L40" s="39" t="inlineStr">
+        <is>
+          <t>Private label juice (own brand)</t>
+        </is>
+      </c>
+      <c r="N40" s="39" t="inlineStr">
+        <is>
+          <t>Wants to import to Malawi; requests WhatsApp contact; Muhammed from Malawi (+265...)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="46" customHeight="1">
       <c r="A41" s="39" t="n">
         <v>37</v>
       </c>
@@ -2386,11 +2594,23 @@
           <t>Product inquiry</t>
         </is>
       </c>
-      <c r="J41" s="39" t="inlineStr"/>
-      <c r="L41" s="39" t="inlineStr"/>
-      <c r="N41" s="39" t="inlineStr"/>
-    </row>
-    <row r="42" ht="30" customHeight="1">
+      <c r="J41" s="39" t="inlineStr">
+        <is>
+          <t>25 MT every 2 months; yearly contract basis with scalable volume</t>
+        </is>
+      </c>
+      <c r="L41" s="39" t="inlineStr">
+        <is>
+          <t>Frozen NFC Lemon Juice (not from concentrate), 100% natural no additives; specs needed Brix, acidity %citric, pH, pulp content, color, shelf life, storage -18C; also Frozen Ginger Juice (NFC/extracted); packaging food-grade HDPE buckets 10-20 L</t>
+        </is>
+      </c>
+      <c r="N41" s="39" t="inlineStr">
+        <is>
+          <t>FOB Alexandria/Damietta/Port Said; CIF Jebel Ali, UAE; immediate shipment; payment advance + balance vs shipping docs (negotiable); docs TDS, COA, ISO/HACCP/Halal; Al Malaky Royal, UAE; Tel 0523525206</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="46" customHeight="1">
       <c r="A42" s="39" t="n">
         <v>38</v>
       </c>
@@ -2422,7 +2642,7 @@
       <c r="L42" s="39" t="inlineStr"/>
       <c r="N42" s="39" t="inlineStr"/>
     </row>
-    <row r="43" ht="30" customHeight="1">
+    <row r="43" ht="46" customHeight="1">
       <c r="A43" s="39" t="n">
         <v>39</v>
       </c>
@@ -2454,7 +2674,7 @@
       <c r="L43" s="39" t="inlineStr"/>
       <c r="N43" s="39" t="inlineStr"/>
     </row>
-    <row r="44" ht="30" customHeight="1">
+    <row r="44" ht="46" customHeight="1">
       <c r="A44" s="39" t="n">
         <v>40</v>
       </c>
@@ -2490,7 +2710,7 @@
       <c r="L44" s="39" t="inlineStr"/>
       <c r="N44" s="39" t="inlineStr"/>
     </row>
-    <row r="45" ht="30" customHeight="1">
+    <row r="45" ht="46" customHeight="1">
       <c r="A45" s="39" t="n">
         <v>41</v>
       </c>
@@ -2523,10 +2743,18 @@
         </is>
       </c>
       <c r="J45" s="39" t="inlineStr"/>
-      <c r="L45" s="39" t="inlineStr"/>
-      <c r="N45" s="39" t="inlineStr"/>
-    </row>
-    <row r="46" ht="30" customHeight="1">
+      <c r="L45" s="39" t="inlineStr">
+        <is>
+          <t>Citrus &amp; fruit concentrates discussed at Gulfood 2026 (no detailed specs given)</t>
+        </is>
+      </c>
+      <c r="N45" s="39" t="inlineStr">
+        <is>
+          <t>Met at Gulfood; copied R&amp;D dept; at this stage not in position to proceed with a purchase order, may revisit later; Samia Dziri, HBC Holding / Hamoud Boualem</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="46" customHeight="1">
       <c r="A46" s="39" t="n">
         <v>42</v>
       </c>
@@ -2559,10 +2787,18 @@
         </is>
       </c>
       <c r="J46" s="39" t="inlineStr"/>
-      <c r="L46" s="39" t="inlineStr"/>
-      <c r="N46" s="39" t="inlineStr"/>
-    </row>
-    <row r="47" ht="30" customHeight="1">
+      <c r="L46" s="39" t="inlineStr">
+        <is>
+          <t>Private label/OEM freeze-dried fruit snacks (strawberry, mango, mixed fruits), bulk &amp; private label; requests MOQ and price list</t>
+        </is>
+      </c>
+      <c r="N46" s="39" t="inlineStr">
+        <is>
+          <t>For export to USA / Amazon US FBA; asks re FDA-compliant labeling, UPC/FNSKU barcoding, export docs &amp; customs, shipping to US freight forwarder/FBA, production availability &amp; lead time; Ghada Abdeen (partner Mr. Alaa met at Gulfood)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="46" customHeight="1">
       <c r="A47" s="39" t="n">
         <v>43</v>
       </c>
@@ -2594,11 +2830,23 @@
           <t>Orange &amp; strawberry concentrate (specs/pricing)</t>
         </is>
       </c>
-      <c r="J47" s="39" t="inlineStr"/>
-      <c r="L47" s="39" t="inlineStr"/>
-      <c r="N47" s="39" t="inlineStr"/>
-    </row>
-    <row r="48" ht="30" customHeight="1">
+      <c r="J47" s="39" t="inlineStr">
+        <is>
+          <t>Orange concentrate 700 MT/yr; strawberry concentrate (without seeds) 100 MT/yr; strawberry concentrate (with seeds) 100 MT/yr</t>
+        </is>
+      </c>
+      <c r="L47" s="39" t="inlineStr">
+        <is>
+          <t>Orange concentrate; strawberry concentrate with and without seeds; aseptic/drums packaging; spec sheets attached (Orange Concentrate, Strawberry Puree, Strawberry Puree with seeds); requests best pricing</t>
+        </is>
+      </c>
+      <c r="N47" s="39" t="inlineStr">
+        <is>
+          <t>Pricing terms EXW &amp; CIF Aqaba (Jordan); met at Gulfood 2026; Ahmad Taha / Abdallah Sweiss, Zain Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="46" customHeight="1">
       <c r="A48" s="39" t="n">
         <v>44</v>
       </c>
@@ -2630,11 +2878,23 @@
           <t>QF fruits &amp; vegetables (Gulfood)</t>
         </is>
       </c>
-      <c r="J48" s="39" t="inlineStr"/>
-      <c r="L48" s="39" t="inlineStr"/>
-      <c r="N48" s="39" t="inlineStr"/>
-    </row>
-    <row r="49" ht="30" customHeight="1">
+      <c r="J48" s="39" t="inlineStr">
+        <is>
+          <t>1 container</t>
+        </is>
+      </c>
+      <c r="L48" s="39" t="inlineStr">
+        <is>
+          <t>IQF fruits &amp; vegetables price list requested; bulk 10KG packaging; packaging: double wall corrugated cartons with polyethylene bags</t>
+        </is>
+      </c>
+      <c r="N48" s="39" t="inlineStr">
+        <is>
+          <t>Follow-up from Gulfood; nina (Qingdao Fresh Dynamic) is supplier sharing prices; WhatsApp 86+15066252086</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="46" customHeight="1">
       <c r="A49" s="39" t="n">
         <v>45</v>
       </c>
@@ -2667,10 +2927,18 @@
         </is>
       </c>
       <c r="J49" s="39" t="inlineStr"/>
-      <c r="L49" s="39" t="inlineStr"/>
-      <c r="N49" s="39" t="inlineStr"/>
-    </row>
-    <row r="50" ht="30" customHeight="1">
+      <c r="L49" s="39" t="inlineStr">
+        <is>
+          <t>Strawberry Puree Concentrate, 8% Brix and 20% Brix, Egypt origin; price per MT requested for both Brix; packaging options (aseptic drums, frozen bags); technical data sheet requested</t>
+        </is>
+      </c>
+      <c r="N49" s="39" t="inlineStr">
+        <is>
+          <t>End buyer in USA via CB Commerce; FDA registration a must, must meet USA MRLs; certs HACCP/ISO/Halal/Organic/FDA; long-term repeat business</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="46" customHeight="1">
       <c r="A50" s="39" t="n">
         <v>46</v>
       </c>
@@ -2707,10 +2975,18 @@
         </is>
       </c>
       <c r="J50" s="39" t="inlineStr"/>
-      <c r="L50" s="39" t="inlineStr"/>
-      <c r="N50" s="39" t="inlineStr"/>
-    </row>
-    <row r="51" ht="30" customHeight="1">
+      <c r="L50" s="39" t="inlineStr">
+        <is>
+          <t>FD (freeze-dried) Strawberry slices and Frozen Strawberry slices; asks if available</t>
+        </is>
+      </c>
+      <c r="N50" s="39" t="inlineStr">
+        <is>
+          <t>Nature Foods Company LTD, Dong Nai, Vietnam; Tel +84903941664</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="46" customHeight="1">
       <c r="A51" s="39" t="n">
         <v>47</v>
       </c>
@@ -2747,10 +3023,18 @@
         </is>
       </c>
       <c r="J51" s="39" t="inlineStr"/>
-      <c r="L51" s="39" t="inlineStr"/>
-      <c r="N51" s="39" t="inlineStr"/>
-    </row>
-    <row r="52" ht="30" customHeight="1">
+      <c r="L51" s="39" t="inlineStr">
+        <is>
+          <t>No specific product/specs; general partnership inquiry for retail/wholesale supply</t>
+        </is>
+      </c>
+      <c r="N51" s="39" t="inlineStr">
+        <is>
+          <t>EDEKA Sudwest Stiftung &amp; Co. KG, Offenburg, Germany; seeking strategic supplier partnership; Tel 015214017665</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="46" customHeight="1">
       <c r="A52" s="39" t="n">
         <v>48</v>
       </c>
@@ -2790,7 +3074,7 @@
       <c r="L52" s="39" t="inlineStr"/>
       <c r="N52" s="39" t="inlineStr"/>
     </row>
-    <row r="53" ht="30" customHeight="1">
+    <row r="53" ht="46" customHeight="1">
       <c r="A53" s="39" t="n">
         <v>49</v>
       </c>
@@ -2822,7 +3106,7 @@
       <c r="L53" s="39" t="inlineStr"/>
       <c r="N53" s="39" t="inlineStr"/>
     </row>
-    <row r="54" ht="30" customHeight="1">
+    <row r="54" ht="46" customHeight="1">
       <c r="A54" s="39" t="n">
         <v>50</v>
       </c>
@@ -2855,10 +3139,18 @@
         </is>
       </c>
       <c r="J54" s="39" t="inlineStr"/>
-      <c r="L54" s="39" t="inlineStr"/>
-      <c r="N54" s="39" t="inlineStr"/>
-    </row>
-    <row r="55" ht="30" customHeight="1">
+      <c r="L54" s="39" t="inlineStr">
+        <is>
+          <t>Custom-cut IQF frozen vegetables (custom cuts); requests available formats, technical specs needed; MOQ and lead times requested</t>
+        </is>
+      </c>
+      <c r="N54" s="39" t="inlineStr">
+        <is>
+          <t>Emirates Flight Catering (Dubai, UAE); flight catering/food service; Tel +971 4 208 6095, Mob +971 56 508 2351; follow-up from Gulfood 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="46" customHeight="1">
       <c r="A55" s="39" t="n">
         <v>51</v>
       </c>
@@ -2886,11 +3178,23 @@
           <t>FD fruits (Strawberry/Mango/Banana, 400-500g, 20ft CIF Rotterdam)</t>
         </is>
       </c>
-      <c r="J55" s="39" t="inlineStr"/>
-      <c r="L55" s="39" t="inlineStr"/>
-      <c r="N55" s="39" t="inlineStr"/>
-    </row>
-    <row r="56" ht="30" customHeight="1">
+      <c r="J55" s="39" t="inlineStr">
+        <is>
+          <t>1x20ft container (10 pallets), first order</t>
+        </is>
+      </c>
+      <c r="L55" s="39" t="inlineStr">
+        <is>
+          <t>FD Strawberry / Mango / Banana, sliced; 400-500 g buckets (branded sticker), palletised</t>
+        </is>
+      </c>
+      <c r="N55" s="39" t="inlineStr">
+        <is>
+          <t>CIF Rotterdam; German sourcing agency buying for client; product brochure &amp; certificates requested</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="46" customHeight="1">
       <c r="A56" s="39" t="n">
         <v>52</v>
       </c>
@@ -2926,11 +3230,23 @@
           <t>Tomato concentrate</t>
         </is>
       </c>
-      <c r="J56" s="39" t="inlineStr"/>
-      <c r="L56" s="39" t="inlineStr"/>
-      <c r="N56" s="39" t="inlineStr"/>
-    </row>
-    <row r="57" ht="30" customHeight="1">
+      <c r="J56" s="39" t="inlineStr">
+        <is>
+          <t>At least 12 full containers annually (estimated)</t>
+        </is>
+      </c>
+      <c r="L56" s="39" t="inlineStr">
+        <is>
+          <t>Tomato concentrate 28/30 Brix (hot break) and 30/32 Brix (hot break); prices needed in all sizes incl retail; bulk/aseptic drums/retail packs</t>
+        </is>
+      </c>
+      <c r="N56" s="39" t="inlineStr">
+        <is>
+          <t>Agile Table SL (Spain) &amp; IMB (US); delivery Busan port/Japan; certs BRC/ISO/Halal/Kosher/Organic; contact +34 676206892</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="46" customHeight="1">
       <c r="A57" s="39" t="n">
         <v>53</v>
       </c>
@@ -2970,7 +3286,7 @@
       <c r="L57" s="39" t="inlineStr"/>
       <c r="N57" s="39" t="inlineStr"/>
     </row>
-    <row r="58" ht="30" customHeight="1">
+    <row r="58" ht="46" customHeight="1">
       <c r="A58" s="39" t="n">
         <v>54</v>
       </c>
@@ -3010,7 +3326,7 @@
       <c r="L58" s="39" t="inlineStr"/>
       <c r="N58" s="39" t="inlineStr"/>
     </row>
-    <row r="59" ht="30" customHeight="1">
+    <row r="59" ht="46" customHeight="1">
       <c r="A59" s="39" t="n">
         <v>55</v>
       </c>
@@ -3047,10 +3363,18 @@
         </is>
       </c>
       <c r="J59" s="39" t="inlineStr"/>
-      <c r="L59" s="39" t="inlineStr"/>
-      <c r="N59" s="39" t="inlineStr"/>
-    </row>
-    <row r="60" ht="30" customHeight="1">
+      <c r="L59" s="39" t="inlineStr">
+        <is>
+          <t>Fresh strawberries for 2026/2027 season, export/processing grade; ready to coordinate specs, quantities, pricing, delivery</t>
+        </is>
+      </c>
+      <c r="N59" s="39" t="inlineStr">
+        <is>
+          <t>Ahmed Sabry offering to supply (potential supplier); asks for required quality standards/certifications; phone 01064476303</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="46" customHeight="1">
       <c r="A60" s="39" t="n">
         <v>56</v>
       </c>
@@ -3087,10 +3411,18 @@
         </is>
       </c>
       <c r="J60" s="39" t="inlineStr"/>
-      <c r="L60" s="39" t="inlineStr"/>
-      <c r="N60" s="39" t="inlineStr"/>
-    </row>
-    <row r="61" ht="30" customHeight="1">
+      <c r="L60" s="39" t="inlineStr">
+        <is>
+          <t>Requests full catalogue and price list; interested in frozen goods, ice cream, chilled and ambient products for distribution</t>
+        </is>
+      </c>
+      <c r="N60" s="39" t="inlineStr">
+        <is>
+          <t>Nickal distributor, Warsaw, Poland; supplies Biedronka, Lidl, Auchan, Intermarche, BP, Shell; wants intro meeting to enter Polish market; Tel 575400582</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="46" customHeight="1">
       <c r="A61" s="39" t="n">
         <v>57</v>
       </c>
@@ -3124,9 +3456,13 @@
       </c>
       <c r="J61" s="39" t="inlineStr"/>
       <c r="L61" s="39" t="inlineStr"/>
-      <c r="N61" s="39" t="inlineStr"/>
-    </row>
-    <row r="62" ht="30" customHeight="1">
+      <c r="N61" s="39" t="inlineStr">
+        <is>
+          <t>Only an out-of-office auto-reply received re Concentrates follow-up (Gulfood 2026); no requirement details provided; contact 8470045903</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="46" customHeight="1">
       <c r="A62" s="39" t="n">
         <v>58</v>
       </c>
@@ -3158,11 +3494,23 @@
           <t>Strawberry &amp; guava concentrate (1 container mixed)</t>
         </is>
       </c>
-      <c r="J62" s="39" t="inlineStr"/>
-      <c r="L62" s="39" t="inlineStr"/>
-      <c r="N62" s="39" t="inlineStr"/>
-    </row>
-    <row r="63" ht="30" customHeight="1">
+      <c r="J62" s="39" t="inlineStr">
+        <is>
+          <t>1 container, mixed items</t>
+        </is>
+      </c>
+      <c r="L62" s="39" t="inlineStr">
+        <is>
+          <t>Strawberry concentrate and guava; requests specifications and best price</t>
+        </is>
+      </c>
+      <c r="N62" s="39" t="inlineStr">
+        <is>
+          <t>Jamil Sabbagh, juice factory in Syria</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="46" customHeight="1">
       <c r="A63" s="39" t="n">
         <v>59</v>
       </c>
@@ -3198,11 +3546,23 @@
           <t>RFQ freeze-dried strawberries</t>
         </is>
       </c>
-      <c r="J63" s="39" t="inlineStr"/>
-      <c r="L63" s="39" t="inlineStr"/>
-      <c r="N63" s="39" t="inlineStr"/>
-    </row>
-    <row r="64" ht="30" customHeight="1">
+      <c r="J63" s="39" t="inlineStr">
+        <is>
+          <t>1 x 20-foot container</t>
+        </is>
+      </c>
+      <c r="L63" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried strawberries (whole and powder); packaging in drums; size/spec 15 x 25; unit &amp; total price, technical data sheet, shelf life/storage requested</t>
+        </is>
+      </c>
+      <c r="N63" s="39" t="inlineStr">
+        <is>
+          <t>Incoterms EXW/FOB/CIF Mersin; destination Mersin Port, Turkey; production/delivery lead time and certifications requested; contact Amal Elhakim 01060333434</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="46" customHeight="1">
       <c r="A64" s="39" t="n">
         <v>60</v>
       </c>
@@ -3236,9 +3596,13 @@
       </c>
       <c r="J64" s="39" t="inlineStr"/>
       <c r="L64" s="39" t="inlineStr"/>
-      <c r="N64" s="39" t="inlineStr"/>
-    </row>
-    <row r="65" ht="30" customHeight="1">
+      <c r="N64" s="39" t="inlineStr">
+        <is>
+          <t>Only auto-reply re Pronat email address change received; no inquiry details</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="46" customHeight="1">
       <c r="A65" s="39" t="n">
         <v>61</v>
       </c>
@@ -3267,10 +3631,18 @@
         </is>
       </c>
       <c r="J65" s="39" t="inlineStr"/>
-      <c r="L65" s="39" t="inlineStr"/>
-      <c r="N65" s="39" t="inlineStr"/>
-    </row>
-    <row r="66" ht="30" customHeight="1">
+      <c r="L65" s="39" t="inlineStr">
+        <is>
+          <t>Juice/fruit concentrates discussed at Gulfood 2026; asks whether MAFI offers organic products from catalogue</t>
+        </is>
+      </c>
+      <c r="N65" s="39" t="inlineStr">
+        <is>
+          <t>Requires EU, USDA or JAS organic certification; Ecoloni Gida (Sakarya, Turkey); contact +90 535 623 54 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="46" customHeight="1">
       <c r="A66" s="39" t="n">
         <v>62</v>
       </c>
@@ -3307,10 +3679,18 @@
         </is>
       </c>
       <c r="J66" s="39" t="inlineStr"/>
-      <c r="L66" s="39" t="inlineStr"/>
-      <c r="N66" s="39" t="inlineStr"/>
-    </row>
-    <row r="67" ht="30" customHeight="1">
+      <c r="L66" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried fruits: FD mango ~2x2 cm pieces, FD pineapple cut into 1/16 pieces, FD strawberries sliced; requests product specifications</t>
+        </is>
+      </c>
+      <c r="N66" s="39" t="inlineStr">
+        <is>
+          <t>Helio S.A., Brochow, Poland; requests delivery terms and offer; Tel 506558283</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="46" customHeight="1">
       <c r="A67" s="39" t="n">
         <v>63</v>
       </c>
@@ -3342,11 +3722,23 @@
           <t>IQF strawberry for France (offer request)</t>
         </is>
       </c>
-      <c r="J67" s="39" t="inlineStr"/>
-      <c r="L67" s="39" t="inlineStr"/>
-      <c r="N67" s="39" t="inlineStr"/>
-    </row>
-    <row r="68" ht="30" customHeight="1">
+      <c r="J67" s="39" t="inlineStr">
+        <is>
+          <t>66,000 KG total (min); 22,000 KG min per shipment</t>
+        </is>
+      </c>
+      <c r="L67" s="39" t="inlineStr">
+        <is>
+          <t>IQF Frozen Strawberry; cardboard box packaging, 20 KG per unit; product specs and availability requested</t>
+        </is>
+      </c>
+      <c r="N67" s="39" t="inlineStr">
+        <is>
+          <t>CFR Marseille, France; first delivery 06/04/2026; include 3% Iberfoods fee in price; Iberfoods commercial office for France market</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="46" customHeight="1">
       <c r="A68" s="39" t="n">
         <v>64</v>
       </c>
@@ -3383,10 +3775,18 @@
         </is>
       </c>
       <c r="J68" s="39" t="inlineStr"/>
-      <c r="L68" s="39" t="inlineStr"/>
-      <c r="N68" s="39" t="inlineStr"/>
-    </row>
-    <row r="69" ht="30" customHeight="1">
+      <c r="L68" s="39" t="inlineStr">
+        <is>
+          <t>IQF Strawberry (context of discussion); no specific requirements provided</t>
+        </is>
+      </c>
+      <c r="N68" s="39" t="inlineStr">
+        <is>
+          <t>Trixy, Longhai Juli Food Co Ltd, China; will revert when there is a need to import IQF strawberry; Tel +86 596-6719777</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="46" customHeight="1">
       <c r="A69" s="39" t="n">
         <v>65</v>
       </c>
@@ -3419,10 +3819,18 @@
         </is>
       </c>
       <c r="J69" s="39" t="inlineStr"/>
-      <c r="L69" s="39" t="inlineStr"/>
-      <c r="N69" s="39" t="inlineStr"/>
-    </row>
-    <row r="70" ht="30" customHeight="1">
+      <c r="L69" s="39" t="inlineStr">
+        <is>
+          <t>Tomato Concentrate (context of discussion); no specific requirements provided yet</t>
+        </is>
+      </c>
+      <c r="N69" s="39" t="inlineStr">
+        <is>
+          <t>Gulf Processing Industries (Sharaf Group), Dubai; forwarded to procurement (Anirudha); their certs HACCP/ISO 22000/FSSC 22000/BRC/Halal/Kosher; M +971 555137949</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="46" customHeight="1">
       <c r="A70" s="39" t="n">
         <v>66</v>
       </c>
@@ -3456,9 +3864,13 @@
       </c>
       <c r="J70" s="39" t="inlineStr"/>
       <c r="L70" s="39" t="inlineStr"/>
-      <c r="N70" s="39" t="inlineStr"/>
-    </row>
-    <row r="71" ht="30" customHeight="1">
+      <c r="N70" s="39" t="inlineStr">
+        <is>
+          <t>No inbound inquiry from this address in folder; only an auto-reply from sanmarzano.com redirecting MAFI's tomato concentrate follow-up to this address</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="46" customHeight="1">
       <c r="A71" s="39" t="n">
         <v>67</v>
       </c>
@@ -3494,11 +3906,23 @@
           <t>Strawberry seed 24 MT</t>
         </is>
       </c>
-      <c r="J71" s="39" t="inlineStr"/>
-      <c r="L71" s="39" t="inlineStr"/>
-      <c r="N71" s="39" t="inlineStr"/>
-    </row>
-    <row r="72" ht="30" customHeight="1">
+      <c r="J71" s="39" t="inlineStr">
+        <is>
+          <t>24 MT</t>
+        </is>
+      </c>
+      <c r="L71" s="39" t="inlineStr">
+        <is>
+          <t>Strawberry seeds (for pressing oil) - not standard fruit product</t>
+        </is>
+      </c>
+      <c r="N71" s="39" t="inlineStr">
+        <is>
+          <t>O&amp;3 Polska Sp. z o.o., Warka, Poland; Tel 506680754</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="46" customHeight="1">
       <c r="A72" s="39" t="n">
         <v>68</v>
       </c>
@@ -3534,11 +3958,23 @@
           <t>Freeze-dried strawberries (20-30 tons; whole/slices/powder)</t>
         </is>
       </c>
-      <c r="J72" s="39" t="inlineStr"/>
-      <c r="L72" s="39" t="inlineStr"/>
-      <c r="N72" s="39" t="inlineStr"/>
-    </row>
-    <row r="73" ht="30" customHeight="1">
+      <c r="J72" s="39" t="inlineStr">
+        <is>
+          <t>20 tons freeze-dried strawberries; quote based on a full container of each shape</t>
+        </is>
+      </c>
+      <c r="L72" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried strawberries: whole, slices, powder; also asks price of IQF strawberries for freeze-drying; requests full quotation</t>
+        </is>
+      </c>
+      <c r="N72" s="39" t="inlineStr">
+        <is>
+          <t>Buyer is CEO of a Czech Republic company; asks for pesticide analyses; notes MAFI starts production Q3 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="46" customHeight="1">
       <c r="A73" s="39" t="n">
         <v>69</v>
       </c>
@@ -3574,7 +4010,7 @@
       <c r="L73" s="39" t="inlineStr"/>
       <c r="N73" s="39" t="inlineStr"/>
     </row>
-    <row r="74" ht="30" customHeight="1">
+    <row r="74" ht="46" customHeight="1">
       <c r="A74" s="39" t="n">
         <v>70</v>
       </c>
@@ -3604,9 +4040,13 @@
       </c>
       <c r="J74" s="39" t="inlineStr"/>
       <c r="L74" s="39" t="inlineStr"/>
-      <c r="N74" s="39" t="inlineStr"/>
-    </row>
-    <row r="75" ht="30" customHeight="1">
+      <c r="N74" s="39" t="inlineStr">
+        <is>
+          <t>Only an auto-reply (out of office 16-22.03); re IQF fruits &amp; vegetables discussed at Gulfood 2026; alt contact Maria Ducheva (maria.ducheva@prowtc.com)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="46" customHeight="1">
       <c r="A75" s="39" t="n">
         <v>71</v>
       </c>
@@ -3643,10 +4083,18 @@
         </is>
       </c>
       <c r="J75" s="39" t="inlineStr"/>
-      <c r="L75" s="39" t="inlineStr"/>
-      <c r="N75" s="39" t="inlineStr"/>
-    </row>
-    <row r="76" ht="30" customHeight="1">
+      <c r="L75" s="39" t="inlineStr">
+        <is>
+          <t>Citrus molasses (byproduct of citrus processing, for biogas) - not standard fruit product; asks if facility produces it</t>
+        </is>
+      </c>
+      <c r="N75" s="39" t="inlineStr">
+        <is>
+          <t>GreenLix, Fredericia, Denmark; biomass/industrial byproduct supplier for biogas; Tel +4571447106</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="46" customHeight="1">
       <c r="A76" s="39" t="n">
         <v>72</v>
       </c>
@@ -3678,11 +4126,23 @@
           <t>Aseptic strawberry puree (drums, CFR UK)</t>
         </is>
       </c>
-      <c r="J76" s="39" t="inlineStr"/>
-      <c r="L76" s="39" t="inlineStr"/>
-      <c r="N76" s="39" t="inlineStr"/>
-    </row>
-    <row r="77" ht="30" customHeight="1">
+      <c r="J76" s="39" t="inlineStr">
+        <is>
+          <t>300 MT strawberry puree (seedless); full container load shipments; spread deliveries</t>
+        </is>
+      </c>
+      <c r="L76" s="39" t="inlineStr">
+        <is>
+          <t>Aseptic strawberry puree, seedless; 0.5mm sieve filter; minimum Brix 6; aseptic 200kg drums</t>
+        </is>
+      </c>
+      <c r="N76" s="39" t="inlineStr">
+        <is>
+          <t>CFR London Gateway; UK market; meet at IFE Food &amp; Drinks London 30 Mar-1 Apr 2026; asks if storage charges apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="46" customHeight="1">
       <c r="A77" s="39" t="n">
         <v>73</v>
       </c>
@@ -3719,10 +4179,18 @@
         </is>
       </c>
       <c r="J77" s="39" t="inlineStr"/>
-      <c r="L77" s="39" t="inlineStr"/>
-      <c r="N77" s="39" t="inlineStr"/>
-    </row>
-    <row r="78" ht="30" customHeight="1">
+      <c r="L77" s="39" t="inlineStr">
+        <is>
+          <t>No fruit products requested; vendor offering stainless steel tanks, food machinery, pasteurizers, CIP, pumps, filling systems</t>
+        </is>
+      </c>
+      <c r="N77" s="39" t="inlineStr">
+        <is>
+          <t>Endulus Krom GmbH, Duisburg, Germany; equipment supplier pitch (not a buyer); Tel +4917667503821</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="46" customHeight="1">
       <c r="A78" s="39" t="n">
         <v>74</v>
       </c>
@@ -3758,11 +4226,23 @@
           <t>FD strawberry slices (price/MOQ)</t>
         </is>
       </c>
-      <c r="J78" s="39" t="inlineStr"/>
-      <c r="L78" s="39" t="inlineStr"/>
-      <c r="N78" s="39" t="inlineStr"/>
-    </row>
-    <row r="79" ht="30" customHeight="1">
+      <c r="J78" s="39" t="inlineStr">
+        <is>
+          <t>Asks MOQ for FD Strawberry slices</t>
+        </is>
+      </c>
+      <c r="L78" s="39" t="inlineStr">
+        <is>
+          <t>FD (freeze-dried) Strawberry slices; asks per-kg price</t>
+        </is>
+      </c>
+      <c r="N78" s="39" t="inlineStr">
+        <is>
+          <t>Chane GmbH, Sandhausen, Germany; Tel 1787811247</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="46" customHeight="1">
       <c r="A79" s="39" t="n">
         <v>75</v>
       </c>
@@ -3798,11 +4278,23 @@
           <t>Orange/lemon/pomegranate concentrate (FOJC Brix 65, 5 containers, Mersin)</t>
         </is>
       </c>
-      <c r="J79" s="39" t="inlineStr"/>
-      <c r="L79" s="39" t="inlineStr"/>
-      <c r="N79" s="39" t="inlineStr"/>
-    </row>
-    <row r="80" ht="30" customHeight="1">
+      <c r="J79" s="39" t="inlineStr">
+        <is>
+          <t>5 containers</t>
+        </is>
+      </c>
+      <c r="L79" s="39" t="inlineStr">
+        <is>
+          <t>Frozen Orange Juice Concentrate (FOJC), Brix 65, aseptic filling in metal drums; also requests orange, lemon &amp; pomegranate concentrate prices and analyses/specs</t>
+        </is>
+      </c>
+      <c r="N79" s="39" t="inlineStr">
+        <is>
+          <t>Delivery port Mersin Seaport, Turkey; WhatsApp/Tel +905070776453; Global Supply Point Gida (Turkey)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="46" customHeight="1">
       <c r="A80" s="39" t="n">
         <v>76</v>
       </c>
@@ -3831,10 +4323,18 @@
         </is>
       </c>
       <c r="J80" s="39" t="inlineStr"/>
-      <c r="L80" s="39" t="inlineStr"/>
-      <c r="N80" s="39" t="inlineStr"/>
-    </row>
-    <row r="81" ht="30" customHeight="1">
+      <c r="L80" s="39" t="inlineStr">
+        <is>
+          <t>CMO (contract manufacturing) of frozen brands: strawberries, artichokes, cauliflower, broccoli, green beans; plus orange concentrate</t>
+        </is>
+      </c>
+      <c r="N80" s="39" t="inlineStr">
+        <is>
+          <t>Kern for Export; asks if MAFI has started operation and about production line availability; mobile +201223955440</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="46" customHeight="1">
       <c r="A81" s="39" t="n">
         <v>77</v>
       </c>
@@ -3870,11 +4370,23 @@
           <t>IQF whole strawberries (1 container, Poti/FOB)</t>
         </is>
       </c>
-      <c r="J81" s="39" t="inlineStr"/>
-      <c r="L81" s="39" t="inlineStr"/>
-      <c r="N81" s="39" t="inlineStr"/>
-    </row>
-    <row r="82" ht="30" customHeight="1">
+      <c r="J81" s="39" t="inlineStr">
+        <is>
+          <t>1 full container IQF whole strawberries (bulk)</t>
+        </is>
+      </c>
+      <c r="L81" s="39" t="inlineStr">
+        <is>
+          <t>IQF whole strawberries, calibrated and uncalibrated (size for each requested); 10 kg bags; for freeze-drying production</t>
+        </is>
+      </c>
+      <c r="N81" s="39" t="inlineStr">
+        <is>
+          <t>Poti Port or FOB; Fergana Exim Agro, Uzbekistan; requests crop year &amp; certificates; tel +998331017330, WhatsApp +998909881122</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="46" customHeight="1">
       <c r="A82" s="39" t="n">
         <v>78</v>
       </c>
@@ -3910,11 +4422,23 @@
           <t>FD slices (mango/banana/peach), strawberry powder/pieces (50kg)</t>
         </is>
       </c>
-      <c r="J82" s="39" t="inlineStr"/>
-      <c r="L82" s="39" t="inlineStr"/>
-      <c r="N82" s="39" t="inlineStr"/>
-    </row>
-    <row r="83" ht="30" customHeight="1">
+      <c r="J82" s="39" t="inlineStr">
+        <is>
+          <t>25 kg and/or 50 kg bulk per item; quote for 50 kg per item requested; MOQ requested</t>
+        </is>
+      </c>
+      <c r="L82" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried: slices (kiwi, lime, strawberry, mango, banana, peach, black olives), whole (raspberry, wild blueberry, cranberry, peas), powder (raspberry, strawberry), pieces (pineapple, apple etc.); 25/50kg foil bag + carton</t>
+        </is>
+      </c>
+      <c r="N82" s="39" t="inlineStr">
+        <is>
+          <t>EXW quote, EU market (also USA); asks EU warehouse, lead time, certs (BRCGS/FSSC22000/HACCP/ISO); Worlds Garden/FRESHZILLA Barcelona; tel 4434828798</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="46" customHeight="1">
       <c r="A83" s="39" t="n">
         <v>79</v>
       </c>
@@ -3947,10 +4471,18 @@
         </is>
       </c>
       <c r="J83" s="39" t="inlineStr"/>
-      <c r="L83" s="39" t="inlineStr"/>
-      <c r="N83" s="39" t="inlineStr"/>
-    </row>
-    <row r="84" ht="30" customHeight="1">
+      <c r="L83" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried berries</t>
+        </is>
+      </c>
+      <c r="N83" s="39" t="inlineStr">
+        <is>
+          <t>Genba Food, Lithuania; wholesaler in the Baltics; seeking a trusted partner in Egypt</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="46" customHeight="1">
       <c r="A84" s="39" t="n">
         <v>80</v>
       </c>
@@ -3983,10 +4515,18 @@
         </is>
       </c>
       <c r="J84" s="39" t="inlineStr"/>
-      <c r="L84" s="39" t="inlineStr"/>
-      <c r="N84" s="39" t="inlineStr"/>
-    </row>
-    <row r="85" ht="30" customHeight="1">
+      <c r="L84" s="39" t="inlineStr">
+        <is>
+          <t>Requests specifications for Strawberry Puree, Mandarin Juice Concentrate, Lemon Juice Concentrate; MAFI sent specs incl Lemon JC 400 GPL/51.5 Brix and 500 GPL/61.15 Brix</t>
+        </is>
+      </c>
+      <c r="N84" s="39" t="inlineStr">
+        <is>
+          <t>Vitmark-Ukraine, Odesa, Ukraine; Head of Procurement; Tel +380 482 344045 / +380 674485428; cc Alina Khmara</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="46" customHeight="1">
       <c r="A85" s="39" t="n">
         <v>81</v>
       </c>
@@ -4022,11 +4562,23 @@
           <t>Samples / product match</t>
         </is>
       </c>
-      <c r="J85" s="39" t="inlineStr"/>
-      <c r="L85" s="39" t="inlineStr"/>
-      <c r="N85" s="39" t="inlineStr"/>
-    </row>
-    <row r="86" ht="30" customHeight="1">
+      <c r="J85" s="39" t="inlineStr">
+        <is>
+          <t>Samples &gt;=0.5 L for lab/technological testing; MOQ requested</t>
+        </is>
+      </c>
+      <c r="L85" s="39" t="inlineStr">
+        <is>
+          <t>Orange juice concentrate with pulp; Brix &gt;=64.0 (up to ~67.0); titratable acidity 4.5-5.8 g/100g; pH 3.3-4.0</t>
+        </is>
+      </c>
+      <c r="N85" s="39" t="inlineStr">
+        <is>
+          <t>JV Chortoq Mineral Water, Tashkent Uzbekistan; asks price, delivery &amp; payment terms, lead time; tel +998909781925; MAFI offered samples Oct 2026 (starts Q3 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="46" customHeight="1">
       <c r="A86" s="39" t="n">
         <v>82</v>
       </c>
@@ -4059,10 +4611,18 @@
         </is>
       </c>
       <c r="J86" s="39" t="inlineStr"/>
-      <c r="L86" s="39" t="inlineStr"/>
-      <c r="N86" s="39" t="inlineStr"/>
-    </row>
-    <row r="87" ht="30" customHeight="1">
+      <c r="L86" s="39" t="inlineStr">
+        <is>
+          <t>General interest in fruit juice concentrates &amp; purees (also essential/edible oils, terpenes, aroma); no specific product/specs given</t>
+        </is>
+      </c>
+      <c r="N86" s="39" t="inlineStr">
+        <is>
+          <t>Independent procurement rep, MTB - More Than Brokers (Brazil); requests to speak with commercial contact; tel +55 48 99197 1513</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="46" customHeight="1">
       <c r="A87" s="39" t="n">
         <v>83</v>
       </c>
@@ -4102,7 +4662,7 @@
       <c r="L87" s="39" t="inlineStr"/>
       <c r="N87" s="39" t="inlineStr"/>
     </row>
-    <row r="88" ht="30" customHeight="1">
+    <row r="88" ht="46" customHeight="1">
       <c r="A88" s="39" t="n">
         <v>84</v>
       </c>
@@ -4123,10 +4683,18 @@
         </is>
       </c>
       <c r="J88" s="39" t="inlineStr"/>
-      <c r="L88" s="39" t="inlineStr"/>
-      <c r="N88" s="39" t="inlineStr"/>
-    </row>
-    <row r="89" ht="30" customHeight="1">
+      <c r="L88" s="39" t="inlineStr">
+        <is>
+          <t>Fruit juice concentrates: guava, mango, strawberry, orange; asks concentration ratio (Brix) and price of each</t>
+        </is>
+      </c>
+      <c r="N88" s="39" t="inlineStr">
+        <is>
+          <t>Inquiry written in Arabic; requesting prices</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="46" customHeight="1">
       <c r="A89" s="39" t="n">
         <v>85</v>
       </c>
@@ -4166,7 +4734,7 @@
       <c r="L89" s="39" t="inlineStr"/>
       <c r="N89" s="39" t="inlineStr"/>
     </row>
-    <row r="90" ht="30" customHeight="1">
+    <row r="90" ht="46" customHeight="1">
       <c r="A90" s="39" t="n">
         <v>86</v>
       </c>
@@ -4198,11 +4766,23 @@
           <t>Purchasing FD fruits (20ft/40ft, FOB/CIF)</t>
         </is>
       </c>
-      <c r="J90" s="39" t="inlineStr"/>
-      <c r="L90" s="39" t="inlineStr"/>
-      <c r="N90" s="39" t="inlineStr"/>
-    </row>
-    <row r="91" ht="30" customHeight="1">
+      <c r="J90" s="39" t="inlineStr">
+        <is>
+          <t>20ft and 40ft containers</t>
+        </is>
+      </c>
+      <c r="L90" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried fruit: Strawberry (whole), Apple, Peach, Raspberry (whole), Mango; 50 gr retail packages and bulk packages</t>
+        </is>
+      </c>
+      <c r="N90" s="39" t="inlineStr">
+        <is>
+          <t>Quote FOB and CIF prices; buyer in Turkiye (Kirlioglu); contact +905521619909</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="46" customHeight="1">
       <c r="A91" s="39" t="n">
         <v>87</v>
       </c>
@@ -4238,11 +4818,23 @@
           <t>Sourcing products in bulk</t>
         </is>
       </c>
-      <c r="J91" s="39" t="inlineStr"/>
-      <c r="L91" s="39" t="inlineStr"/>
-      <c r="N91" s="39" t="inlineStr"/>
-    </row>
-    <row r="92" ht="30" customHeight="1">
+      <c r="J91" s="39" t="inlineStr">
+        <is>
+          <t>Bulk quantity (unspecified)</t>
+        </is>
+      </c>
+      <c r="L91" s="39" t="inlineStr">
+        <is>
+          <t>Various products in bulk; requests product catalogue, pricing and availability</t>
+        </is>
+      </c>
+      <c r="N91" s="39" t="inlineStr">
+        <is>
+          <t>Partnership opportunity; delivery to Santiago, Chile; Bureauveritas; Tel 990354287</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="46" customHeight="1">
       <c r="A92" s="39" t="n">
         <v>88</v>
       </c>
@@ -4278,11 +4870,23 @@
           <t>Procurement inquiry</t>
         </is>
       </c>
-      <c r="J92" s="39" t="inlineStr"/>
-      <c r="L92" s="39" t="inlineStr"/>
-      <c r="N92" s="39" t="inlineStr"/>
-    </row>
-    <row r="93" ht="30" customHeight="1">
+      <c r="J92" s="39" t="inlineStr">
+        <is>
+          <t>MOQ requested per product/packaging size (not specified)</t>
+        </is>
+      </c>
+      <c r="L92" s="39" t="inlineStr">
+        <is>
+          <t>Purees, concentrates, IQF/bulk frozen fruit (e.g. IQF pomegranate, strawberries) for smoothies/juices/spreads; specs Brix, pH, ingredient declaration, size/grade, sugar, origin, freezing method, packaging; sample + bulk price in EUR/USD</t>
+        </is>
+      </c>
+      <c r="N92" s="39" t="inlineStr">
+        <is>
+          <t>Delivery to Thessaloniki Port, Greece; Incoterm to be defined; payment terms; certs ISO/HACCP/FSSC22000/Organic/Kosher/Halal; lead time; P Gkotzaridis &amp; Co, Greece</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="46" customHeight="1">
       <c r="A93" s="39" t="n">
         <v>89</v>
       </c>
@@ -4319,10 +4923,18 @@
         </is>
       </c>
       <c r="J93" s="39" t="inlineStr"/>
-      <c r="L93" s="39" t="inlineStr"/>
-      <c r="N93" s="39" t="inlineStr"/>
-    </row>
-    <row r="94" ht="30" customHeight="1">
+      <c r="L93" s="39" t="inlineStr">
+        <is>
+          <t>Natural frozen lemon juice (100% freshly squeezed, frozen at -40C then stored -18C); requesting spec, packaging and price info</t>
+        </is>
+      </c>
+      <c r="N93" s="39" t="inlineStr">
+        <is>
+          <t>Buyer Lemonera/UJ Group, Turkey; plans to visit Egypt to meet suppliers, requests office/factory addresses; T +90 212 9860636/+1 713 7771000, M +90 532 5972721</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="46" customHeight="1">
       <c r="A94" s="39" t="n">
         <v>90</v>
       </c>
@@ -4354,11 +4966,23 @@
           <t>Lemon juice concentrate cloudy/clear 400-500 gpl (2026 demand)</t>
         </is>
       </c>
-      <c r="J94" s="39" t="inlineStr"/>
-      <c r="L94" s="39" t="inlineStr"/>
-      <c r="N94" s="39" t="inlineStr"/>
-    </row>
-    <row r="95" ht="30" customHeight="1">
+      <c r="J94" s="39" t="inlineStr">
+        <is>
+          <t>2026 annual demand (securing volumes for 2026)</t>
+        </is>
+      </c>
+      <c r="L94" s="39" t="inlineStr">
+        <is>
+          <t>Lemon juice concentrate cloudy 400/500 gpl; Lemon juice concentrate clear 400/500 gpl</t>
+        </is>
+      </c>
+      <c r="N94" s="39" t="inlineStr">
+        <is>
+          <t>Requests best price FOB basis, specs and estimated lead time; buyer Pilmifresh</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="46" customHeight="1">
       <c r="A95" s="39" t="n">
         <v>91</v>
       </c>
@@ -4394,7 +5018,7 @@
       <c r="L95" s="39" t="inlineStr"/>
       <c r="N95" s="39" t="inlineStr"/>
     </row>
-    <row r="96" ht="30" customHeight="1">
+    <row r="96" ht="46" customHeight="1">
       <c r="A96" s="39" t="n">
         <v>92</v>
       </c>
@@ -4430,11 +5054,23 @@
           <t>Sales inquiry</t>
         </is>
       </c>
-      <c r="J96" s="39" t="inlineStr"/>
-      <c r="L96" s="39" t="inlineStr"/>
-      <c r="N96" s="39" t="inlineStr"/>
-    </row>
-    <row r="97" ht="30" customHeight="1">
+      <c r="J96" s="39" t="inlineStr">
+        <is>
+          <t>MOQ requested (not specified); samples requested</t>
+        </is>
+      </c>
+      <c r="L96" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried fruits: Mango (chunks/slices), Strawberry (whole/slices), Banana (slices), Kiwi (slices); requests catalog and wholesale price list</t>
+        </is>
+      </c>
+      <c r="N96" s="39" t="inlineStr">
+        <is>
+          <t>Elreefy Trading Co., Giza, Egypt; contact tel 01158300643 / 01061498589</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="46" customHeight="1">
       <c r="A97" s="39" t="n">
         <v>93</v>
       </c>
@@ -4471,10 +5107,18 @@
         </is>
       </c>
       <c r="J97" s="39" t="inlineStr"/>
-      <c r="L97" s="39" t="inlineStr"/>
-      <c r="N97" s="39" t="inlineStr"/>
-    </row>
-    <row r="98" ht="30" customHeight="1">
+      <c r="L97" s="39" t="inlineStr">
+        <is>
+          <t>Requests full brochure for all upcoming products and a quotation if possible</t>
+        </is>
+      </c>
+      <c r="N97" s="39" t="inlineStr">
+        <is>
+          <t>Dubai, UAE; Tel +971503409475; MAFI replied with brochure &amp; company profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="46" customHeight="1">
       <c r="A98" s="39" t="n">
         <v>94</v>
       </c>
@@ -4511,10 +5155,18 @@
         </is>
       </c>
       <c r="J98" s="39" t="inlineStr"/>
-      <c r="L98" s="39" t="inlineStr"/>
-      <c r="N98" s="39" t="inlineStr"/>
-    </row>
-    <row r="99" ht="30" customHeight="1">
+      <c r="L98" s="39" t="inlineStr">
+        <is>
+          <t>Looking for NFC orange juice</t>
+        </is>
+      </c>
+      <c r="N98" s="39" t="inlineStr">
+        <is>
+          <t>Andros, France; plans to visit Egypt in March, asks to visit on the 11th; Tel 0033620730939</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="46" customHeight="1">
       <c r="A99" s="39" t="n">
         <v>95</v>
       </c>
@@ -4551,10 +5203,18 @@
         </is>
       </c>
       <c r="J99" s="39" t="inlineStr"/>
-      <c r="L99" s="39" t="inlineStr"/>
-      <c r="N99" s="39" t="inlineStr"/>
-    </row>
-    <row r="100" ht="30" customHeight="1">
+      <c r="L99" s="39" t="inlineStr">
+        <is>
+          <t>Concentrated fruit juices and purees: peach, cherry, apricot, apple, etc.; requests product specifications and indicative price</t>
+        </is>
+      </c>
+      <c r="N99" s="39" t="inlineStr">
+        <is>
+          <t>PROGRESS (Frutonanny), baby food producer, Moscow, Russia; Tel +79264121460</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="46" customHeight="1">
       <c r="A100" s="39" t="n">
         <v>96</v>
       </c>
@@ -4590,11 +5250,23 @@
           <t>Sweet potato varieties / EU export &amp; chips line</t>
         </is>
       </c>
-      <c r="J100" s="39" t="inlineStr"/>
-      <c r="L100" s="39" t="inlineStr"/>
-      <c r="N100" s="39" t="inlineStr"/>
-    </row>
-    <row r="101" ht="30" customHeight="1">
+      <c r="J100" s="39" t="inlineStr">
+        <is>
+          <t>Reference: Peru exports ~80,000-100,000 t/yr and Chile ~15,000-25,000 t/yr sweet potatoes to EU</t>
+        </is>
+      </c>
+      <c r="L100" s="39" t="inlineStr">
+        <is>
+          <t>Sweet potato varieties (Japanese Satsumaimo/Murasaki, purple-flesh Okinawan, white-flesh processing types) for IQF/chips; partnership to cultivate in Egypt and export to EU</t>
+        </is>
+      </c>
+      <c r="N100" s="39" t="inlineStr">
+        <is>
+          <t>Destination EU (Germany, Spain, France, Netherlands); proposes technical call/pilot phase; Uniya Chile spa; phone +56 9 3414 3633</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="46" customHeight="1">
       <c r="A101" s="39" t="n">
         <v>97</v>
       </c>
@@ -4634,7 +5306,7 @@
       <c r="L101" s="39" t="inlineStr"/>
       <c r="N101" s="39" t="inlineStr"/>
     </row>
-    <row r="102" ht="30" customHeight="1">
+    <row r="102" ht="46" customHeight="1">
       <c r="A102" s="39" t="n">
         <v>98</v>
       </c>
@@ -4674,7 +5346,7 @@
       <c r="L102" s="39" t="inlineStr"/>
       <c r="N102" s="39" t="inlineStr"/>
     </row>
-    <row r="103" ht="30" customHeight="1">
+    <row r="103" ht="46" customHeight="1">
       <c r="A103" s="39" t="n">
         <v>99</v>
       </c>
@@ -4710,11 +5382,23 @@
           <t>Import inquiry</t>
         </is>
       </c>
-      <c r="J103" s="39" t="inlineStr"/>
-      <c r="L103" s="39" t="inlineStr"/>
-      <c r="N103" s="39" t="inlineStr"/>
-    </row>
-    <row r="104" ht="30" customHeight="1">
+      <c r="J103" s="39" t="inlineStr">
+        <is>
+          <t>1x 20ft FCL or 1x 40ft FCL</t>
+        </is>
+      </c>
+      <c r="L103" s="39" t="inlineStr">
+        <is>
+          <t>NFC Orange Juice; packing 200 L drums or 1000 L IBC tanks; requests FOB prices, product photos, spec sheet (broker takes 5% commission on FOB)</t>
+        </is>
+      </c>
+      <c r="N103" s="39" t="inlineStr">
+        <is>
+          <t>FOB for Brazil market; needs port of loading, container load 20/40ft, ETD, payment terms, price validity; HR Broker, Maceio, Brazil; Tel 9373399905</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="46" customHeight="1">
       <c r="A104" s="39" t="n">
         <v>100</v>
       </c>
@@ -4747,10 +5431,18 @@
         </is>
       </c>
       <c r="J104" s="39" t="inlineStr"/>
-      <c r="L104" s="39" t="inlineStr"/>
-      <c r="N104" s="39" t="inlineStr"/>
-    </row>
-    <row r="105" ht="30" customHeight="1">
+      <c r="L104" s="39" t="inlineStr">
+        <is>
+          <t>Rehydrated prunes, with pit and pitted, for industrial fruit processing (purees, fillings, jams) - supplier offer, not buyer request</t>
+        </is>
+      </c>
+      <c r="N104" s="39" t="inlineStr">
+        <is>
+          <t>Originia Foods / SAMCA Group, Spain; requests intro call; contact +34 976160188, +34 690092156, Ana Arnal</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="46" customHeight="1">
       <c r="A105" s="39" t="n">
         <v>101</v>
       </c>
@@ -4786,11 +5478,23 @@
           <t>Supply fresh/IQF strawberries (300 tons, FDA)</t>
         </is>
       </c>
-      <c r="J105" s="39" t="inlineStr"/>
-      <c r="L105" s="39" t="inlineStr"/>
-      <c r="N105" s="39" t="inlineStr"/>
-    </row>
-    <row r="106" ht="30" customHeight="1">
+      <c r="J105" s="39" t="inlineStr">
+        <is>
+          <t>300 tons</t>
+        </is>
+      </c>
+      <c r="L105" s="39" t="inlineStr">
+        <is>
+          <t>Strawberries ready for freezing; FDA-tested and dried (freeze-dried) strawberries</t>
+        </is>
+      </c>
+      <c r="N105" s="39" t="inlineStr">
+        <is>
+          <t>Arabic inquiry (Allian for Agricultural Supplies); asks delivery timing and contracting method; contact 01007075225</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="46" customHeight="1">
       <c r="A106" s="39" t="n">
         <v>102</v>
       </c>
@@ -4822,11 +5526,23 @@
           <t>Supply fresh strawberries</t>
         </is>
       </c>
-      <c r="J106" s="39" t="inlineStr"/>
-      <c r="L106" s="39" t="inlineStr"/>
-      <c r="N106" s="39" t="inlineStr"/>
-    </row>
-    <row r="107" ht="30" customHeight="1">
+      <c r="J106" s="39" t="inlineStr">
+        <is>
+          <t>Required quantities (unspecified)</t>
+        </is>
+      </c>
+      <c r="L106" s="39" t="inlineStr">
+        <is>
+          <t>Direct supply of fruits (general); no specific product/specs given</t>
+        </is>
+      </c>
+      <c r="N106" s="39" t="inlineStr">
+        <is>
+          <t>Generic collaboration/supply proposal; wants to discuss technical and commercial details; contact 01013579935 (Ahmed Ali)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="46" customHeight="1">
       <c r="A107" s="39" t="n">
         <v>103</v>
       </c>
@@ -4859,10 +5575,18 @@
         </is>
       </c>
       <c r="J107" s="39" t="inlineStr"/>
-      <c r="L107" s="39" t="inlineStr"/>
-      <c r="N107" s="39" t="inlineStr"/>
-    </row>
-    <row r="108" ht="30" customHeight="1">
+      <c r="L107" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried products (full range requested); requests pricing and MOQ, packaging info</t>
+        </is>
+      </c>
+      <c r="N107" s="39" t="inlineStr">
+        <is>
+          <t>Export to Morocco; requests export conditions, quality certifications, catalogues/specs/samples; Morocco SAULE; contact +212662680881 (Leila Khedji, CEO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="46" customHeight="1">
       <c r="A108" s="39" t="n">
         <v>104</v>
       </c>
@@ -4898,7 +5622,7 @@
       <c r="L108" s="39" t="inlineStr"/>
       <c r="N108" s="39" t="inlineStr"/>
     </row>
-    <row r="109" ht="30" customHeight="1">
+    <row r="109" ht="46" customHeight="1">
       <c r="A109" s="39" t="n">
         <v>105</v>
       </c>
@@ -4931,10 +5655,18 @@
         </is>
       </c>
       <c r="J109" s="39" t="inlineStr"/>
-      <c r="L109" s="39" t="inlineStr"/>
-      <c r="N109" s="39" t="inlineStr"/>
-    </row>
-    <row r="110" ht="30" customHeight="1">
+      <c r="L109" s="39" t="inlineStr">
+        <is>
+          <t>Seeks organic fruit seeds for vegetable oil production: organic Strawberry, Raspberry, Black currant, Blueberry seeds (not standard fruit products)</t>
+        </is>
+      </c>
+      <c r="N109" s="39" t="inlineStr">
+        <is>
+          <t>Oleador GmbH, Hannover, Germany; reply to MAFI Gulfood 2026 outreach; Tel +49 511 676559-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="46" customHeight="1">
       <c r="A110" s="39" t="n">
         <v>106</v>
       </c>
@@ -4962,11 +5694,23 @@
           <t>FD strawberries (granules) 7 tons - export to China</t>
         </is>
       </c>
-      <c r="J110" s="39" t="inlineStr"/>
-      <c r="L110" s="39" t="inlineStr"/>
-      <c r="N110" s="39" t="inlineStr"/>
-    </row>
-    <row r="111" ht="30" customHeight="1">
+      <c r="J110" s="39" t="inlineStr">
+        <is>
+          <t>7 tons</t>
+        </is>
+      </c>
+      <c r="L110" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried strawberries (granules); Grade: premium food grade</t>
+        </is>
+      </c>
+      <c r="N110" s="39" t="inlineStr">
+        <is>
+          <t>Export to China; requests availability, price quotation and available certifications; Garden Guru; contact 01066650873 (Dr Nesrine Hammady)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="46" customHeight="1">
       <c r="A111" s="39" t="n">
         <v>107</v>
       </c>
@@ -5006,7 +5750,7 @@
       <c r="L111" s="39" t="inlineStr"/>
       <c r="N111" s="39" t="inlineStr"/>
     </row>
-    <row r="112" ht="30" customHeight="1">
+    <row r="112" ht="46" customHeight="1">
       <c r="A112" s="39" t="n">
         <v>108</v>
       </c>
@@ -5046,7 +5790,7 @@
       <c r="L112" s="39" t="inlineStr"/>
       <c r="N112" s="39" t="inlineStr"/>
     </row>
-    <row r="113" ht="30" customHeight="1">
+    <row r="113" ht="46" customHeight="1">
       <c r="A113" s="39" t="n">
         <v>109</v>
       </c>
@@ -5082,7 +5826,7 @@
       <c r="L113" s="39" t="inlineStr"/>
       <c r="N113" s="39" t="inlineStr"/>
     </row>
-    <row r="114" ht="30" customHeight="1">
+    <row r="114" ht="46" customHeight="1">
       <c r="A114" s="39" t="n">
         <v>110</v>
       </c>
@@ -5120,9 +5864,13 @@
       </c>
       <c r="J114" s="39" t="inlineStr"/>
       <c r="L114" s="39" t="inlineStr"/>
-      <c r="N114" s="39" t="inlineStr"/>
-    </row>
-    <row r="115" ht="30" customHeight="1">
+      <c r="N114" s="39" t="inlineStr">
+        <is>
+          <t>General intro via website contact form; wants to discuss business opportunities for REWE Germany; REWE Far East Ltd, Istanbul Turkey; Tel +905423193883</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="46" customHeight="1">
       <c r="A115" s="39" t="n">
         <v>111</v>
       </c>
@@ -5160,9 +5908,13 @@
       </c>
       <c r="J115" s="39" t="inlineStr"/>
       <c r="L115" s="39" t="inlineStr"/>
-      <c r="N115" s="39" t="inlineStr"/>
-    </row>
-    <row r="116" ht="30" customHeight="1">
+      <c r="N115" s="39" t="inlineStr">
+        <is>
+          <t>Not a buyer - Ovorider is Smurfit WestRock agent in ME pitching Bag-in-Box liquid packaging (juices/sauces); requests meeting at Gulfood; Dubai UAE; Tel +962790389890</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="46" customHeight="1">
       <c r="A116" s="39" t="n">
         <v>112</v>
       </c>
@@ -5194,11 +5946,23 @@
           <t>Representation &amp; sales for Brazil</t>
         </is>
       </c>
-      <c r="J116" s="39" t="inlineStr"/>
-      <c r="L116" s="39" t="inlineStr"/>
-      <c r="N116" s="39" t="inlineStr"/>
-    </row>
-    <row r="117" ht="30" customHeight="1">
+      <c r="J116" s="39" t="inlineStr">
+        <is>
+          <t>Has supplied 10,000+ tons strawberries; multiple containers; wants exclusive Brazil representation</t>
+        </is>
+      </c>
+      <c r="L116" s="39" t="inlineStr">
+        <is>
+          <t>IQF strawberries, freeze-dried strawberries, purees and concentrates line</t>
+        </is>
+      </c>
+      <c r="N116" s="39" t="inlineStr">
+        <is>
+          <t>Importer/distributor Frutas do Mundo Ltda, Brazil; Ricardo Pascal; seeks new products/exclusive rep for Brazil; WhatsApp +5551981187269, +5548998491012</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="46" customHeight="1">
       <c r="A117" s="39" t="n">
         <v>113</v>
       </c>
@@ -5234,11 +5998,23 @@
           <t>Processing company - sourcing inquiry</t>
         </is>
       </c>
-      <c r="J117" s="39" t="inlineStr"/>
-      <c r="L117" s="39" t="inlineStr"/>
-      <c r="N117" s="39" t="inlineStr"/>
-    </row>
-    <row r="118" ht="30" customHeight="1">
+      <c r="J117" s="39" t="inlineStr">
+        <is>
+          <t>Asking MOQ; volume/long-term contract discounts requested</t>
+        </is>
+      </c>
+      <c r="L117" s="39" t="inlineStr">
+        <is>
+          <t>NFC (Not-From-Concentrate) orange juice; asks Brix/acidity, pasteurization, packaging (aseptic bag-in-box, PET), shelf life; price per MT in USD</t>
+        </is>
+      </c>
+      <c r="N117" s="39" t="inlineStr">
+        <is>
+          <t>Incoterms FOB/CIF requested; certs ISO/HACCP/organic/Fair Trade; wants samples, facility location, lead time; MJC co, St Petersburg Russia; Tel +79817146772</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="46" customHeight="1">
       <c r="A118" s="39" t="n">
         <v>114</v>
       </c>
@@ -5275,10 +6051,18 @@
         </is>
       </c>
       <c r="J118" s="39" t="inlineStr"/>
-      <c r="L118" s="39" t="inlineStr"/>
-      <c r="N118" s="39" t="inlineStr"/>
-    </row>
-    <row r="119" ht="30" customHeight="1">
+      <c r="L118" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried strawberries</t>
+        </is>
+      </c>
+      <c r="N118" s="39" t="inlineStr">
+        <is>
+          <t>Maya Holling, Badger Ingredients/Ingredient Logistics (US); Office +1 480-404-9539, Mobile +1 480-639-8982</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="46" customHeight="1">
       <c r="A119" s="39" t="n">
         <v>115</v>
       </c>
@@ -5306,11 +6090,23 @@
           <t>Whole FD strawberries (Turkish client)</t>
         </is>
       </c>
-      <c r="J119" s="39" t="inlineStr"/>
-      <c r="L119" s="39" t="inlineStr"/>
-      <c r="N119" s="39" t="inlineStr"/>
-    </row>
-    <row r="120" ht="30" customHeight="1">
+      <c r="J119" s="39" t="inlineStr">
+        <is>
+          <t>Quantities to be agreed at meeting</t>
+        </is>
+      </c>
+      <c r="L119" s="39" t="inlineStr">
+        <is>
+          <t>Whole freeze-dried strawberries</t>
+        </is>
+      </c>
+      <c r="N119" s="39" t="inlineStr">
+        <is>
+          <t>City Run Group, export services, Sadat City; sourcing for a Turkish client visiting Egypt 27th-29th; requests meeting to agree quantities/prices; Mahran Yousof CFO +201114449383</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="46" customHeight="1">
       <c r="A120" s="39" t="n">
         <v>116</v>
       </c>
@@ -5342,11 +6138,23 @@
           <t>FD fruit private label/OEM export to US</t>
         </is>
       </c>
-      <c r="J120" s="39" t="inlineStr"/>
-      <c r="L120" s="39" t="inlineStr"/>
-      <c r="N120" s="39" t="inlineStr"/>
-    </row>
-    <row r="121" ht="30" customHeight="1">
+      <c r="J120" s="39" t="inlineStr">
+        <is>
+          <t>Asking MOQ for private label freeze-dried products</t>
+        </is>
+      </c>
+      <c r="L120" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried fruit snacks - strawberry, mango, mixed fruits; private label/OEM; requests price list (bulk and private label)</t>
+        </is>
+      </c>
+      <c r="N120" s="39" t="inlineStr">
+        <is>
+          <t>Export to US/Amazon FBA; FDA-compliant labeling, UPC/FNSKU barcoding, export docs/customs, ship to US forwarder/FBA; asks lead time &amp; production availability; US startup managed from UAE; Tel +971562021745</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="46" customHeight="1">
       <c r="A121" s="39" t="n">
         <v>117</v>
       </c>
@@ -5382,7 +6190,7 @@
       <c r="L121" s="39" t="inlineStr"/>
       <c r="N121" s="39" t="inlineStr"/>
     </row>
-    <row r="122" ht="30" customHeight="1">
+    <row r="122" ht="46" customHeight="1">
       <c r="A122" s="39" t="n">
         <v>118</v>
       </c>
@@ -5414,7 +6222,7 @@
       <c r="L122" s="39" t="inlineStr"/>
       <c r="N122" s="39" t="inlineStr"/>
     </row>
-    <row r="123" ht="30" customHeight="1">
+    <row r="123" ht="46" customHeight="1">
       <c r="A123" s="39" t="n">
         <v>119</v>
       </c>
@@ -5447,10 +6255,18 @@
         </is>
       </c>
       <c r="J123" s="39" t="inlineStr"/>
-      <c r="L123" s="39" t="inlineStr"/>
-      <c r="N123" s="39" t="inlineStr"/>
-    </row>
-    <row r="124" ht="30" customHeight="1">
+      <c r="L123" s="39" t="inlineStr">
+        <is>
+          <t>Requests explanation of products and prices plus packaging</t>
+        </is>
+      </c>
+      <c r="N123" s="39" t="inlineStr">
+        <is>
+          <t>Mohamad Khalil, Lagos, Nigeria; general product/price inquiry</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="46" customHeight="1">
       <c r="A124" s="39" t="n">
         <v>120</v>
       </c>
@@ -5482,11 +6298,23 @@
           <t>FD strawberries 50 MT export to China (CIF Shanghai)</t>
         </is>
       </c>
-      <c r="J124" s="39" t="inlineStr"/>
-      <c r="L124" s="39" t="inlineStr"/>
-      <c r="N124" s="39" t="inlineStr"/>
-    </row>
-    <row r="125" ht="30" customHeight="1">
+      <c r="J124" s="39" t="inlineStr">
+        <is>
+          <t>50 metric tons for export to China</t>
+        </is>
+      </c>
+      <c r="L124" s="39" t="inlineStr">
+        <is>
+          <t>1) FD strawberries whole, premium food grade, moisture &lt;=5% (target &lt;=3%), 10kg carton w/ 4x2.5kg inner bags; 2) FD strawberry powder 100% (no sugar/carriers), moisture &lt;=4%; FDA/USDA compliant</t>
+        </is>
+      </c>
+      <c r="N124" s="39" t="inlineStr">
+        <is>
+          <t>CIF Shanghai; certs HACCP/ISO/BRC/Organic, COA, heavy metals &amp; pesticide testing; asks MOQ/container plan, lead time, payment terms, samples (partner in China till 8 Jan); Garden Guru, Cairo; Taha Azouz +201114200008</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="46" customHeight="1">
       <c r="A125" s="39" t="n">
         <v>121</v>
       </c>
@@ -5522,7 +6350,7 @@
       <c r="L125" s="39" t="inlineStr"/>
       <c r="N125" s="39" t="inlineStr"/>
     </row>
-    <row r="126" ht="30" customHeight="1">
+    <row r="126" ht="46" customHeight="1">
       <c r="A126" s="39" t="n">
         <v>122</v>
       </c>
@@ -5555,10 +6383,18 @@
         </is>
       </c>
       <c r="J126" s="39" t="inlineStr"/>
-      <c r="L126" s="39" t="inlineStr"/>
-      <c r="N126" s="39" t="inlineStr"/>
-    </row>
-    <row r="127" ht="30" customHeight="1">
+      <c r="L126" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried strawberries, whole, 15-25 mm, preferably round form (not prolongated); quality (taste/appearance); requests quote and product specs</t>
+        </is>
+      </c>
+      <c r="N126" s="39" t="inlineStr">
+        <is>
+          <t>FCA price and CFR Hamburg requested; must comply with EU legislation (pesticides, heavy metals contaminants); Fruzbi Ukraine LLC for EU partner; wants meeting at FI Europe 2025; Anatolii Kondratenko +380931352755, dir Max +380673103857</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="46" customHeight="1">
       <c r="A127" s="39" t="n">
         <v>123</v>
       </c>
@@ -5596,9 +6432,13 @@
       </c>
       <c r="J127" s="39" t="inlineStr"/>
       <c r="L127" s="39" t="inlineStr"/>
-      <c r="N127" s="39" t="inlineStr"/>
-    </row>
-    <row r="128" ht="30" customHeight="1">
+      <c r="N127" s="39" t="inlineStr">
+        <is>
+          <t>Not a buyer - Egyptian supplier (Anwar Moussa, Nubaria/Beheira) offering to supply fresh/frozen produce &amp; citrus to MAFI's Sadat City concentrate factory; Tel 01014147590, 01555087590; MAFI replied will cooperate once plant starts</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="46" customHeight="1">
       <c r="A128" s="39" t="n">
         <v>124</v>
       </c>
@@ -5630,11 +6470,23 @@
           <t>FD strawberries sliced 10,000 kg (offer request)</t>
         </is>
       </c>
-      <c r="J128" s="39" t="inlineStr"/>
-      <c r="L128" s="39" t="inlineStr"/>
-      <c r="N128" s="39" t="inlineStr"/>
-    </row>
-    <row r="129" ht="30" customHeight="1">
+      <c r="J128" s="39" t="inlineStr">
+        <is>
+          <t>10,000 kg</t>
+        </is>
+      </c>
+      <c r="L128" s="39" t="inlineStr">
+        <is>
+          <t>Conventional FD strawberries, sliced; residual moisture max 5%, powder content max 5%, DGHM micro standards, no irradiated/GMO raw materials, metal-detector/X-ray foreign-body control; organic option queried</t>
+        </is>
+      </c>
+      <c r="N128" s="39" t="inlineStr">
+        <is>
+          <t>Requests MOQ &amp; volume-based price tiers; will only buy with intact certification chain - asks for IFS / BRC / FSSC 22000</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="46" customHeight="1">
       <c r="A129" s="39" t="n">
         <v>125</v>
       </c>
@@ -5666,11 +6518,23 @@
           <t>Fruit waste/seeds after puree production (2026-28)</t>
         </is>
       </c>
-      <c r="J129" s="39" t="inlineStr"/>
-      <c r="L129" s="39" t="inlineStr"/>
-      <c r="N129" s="39" t="inlineStr"/>
-    </row>
-    <row r="130" ht="30" customHeight="1">
+      <c r="J129" s="39" t="inlineStr">
+        <is>
+          <t>Single pallets up to FTL refrigerated (40 pallets = 160 drums); ~10 MT strawberry seed waste per 100 MT puree</t>
+        </is>
+      </c>
+      <c r="L129" s="39" t="inlineStr">
+        <is>
+          <t>Frozen fruit waste/seeds after puree/concentrate production - strawberry (high seed content), blackcurrant, passion fruit, kiwi, fig, prickly pear, all organic; packed in used drums/box pallets</t>
+        </is>
+      </c>
+      <c r="N129" s="39" t="inlineStr">
+        <is>
+          <t>Long-term cooperation 2026/27/28; more seeds = higher price; wants Teams meeting; sent sample photos; GreenField Sp z o.o., Warsaw Poland; Pawel Gucajtis +48 502 170 343</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="46" customHeight="1">
       <c r="A130" s="39" t="n">
         <v>126</v>
       </c>
@@ -5702,11 +6566,23 @@
           <t>Orange Juice Concentrate (demand 200MT/month; wants to be Chinese representative)</t>
         </is>
       </c>
-      <c r="J130" s="39" t="inlineStr"/>
-      <c r="L130" s="39" t="inlineStr"/>
-      <c r="N130" s="39" t="inlineStr"/>
-    </row>
-    <row r="131" ht="30" customHeight="1">
+      <c r="J130" s="39" t="inlineStr">
+        <is>
+          <t>Can sell 200 MT per month; wants to be Chinese representative</t>
+        </is>
+      </c>
+      <c r="L130" s="39" t="inlineStr">
+        <is>
+          <t>Orange Juice Concentrate; asks if blended or pure concentrate; requests COA</t>
+        </is>
+      </c>
+      <c r="N130" s="39" t="inlineStr">
+        <is>
+          <t>China importer Far Way Agro (Shaanxi); imports citrus from Egypt &amp; OJC from S.Africa/Brazil/Spain; asks current OJC stock (Egyptian oranges start Dec); Darren Yang +86 132 8929 9418</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="46" customHeight="1">
       <c r="A131" s="39" t="n">
         <v>127</v>
       </c>
@@ -5743,10 +6619,18 @@
         </is>
       </c>
       <c r="J131" s="39" t="inlineStr"/>
-      <c r="L131" s="39" t="inlineStr"/>
-      <c r="N131" s="39" t="inlineStr"/>
-    </row>
-    <row r="132" ht="30" customHeight="1">
+      <c r="L131" s="39" t="inlineStr">
+        <is>
+          <t>Freeze-dried (FD) strawberries; requests specifications and samples</t>
+        </is>
+      </c>
+      <c r="N131" s="39" t="inlineStr">
+        <is>
+          <t>Trawosa AG, St Gallen Switzerland; Michael Lang, Product Manager; already has many customers for FD strawberry products; open to cooperation, asked when production starts (MAFI: Q1/Q2 2026); Tel +41 78 882 04 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="46" customHeight="1">
       <c r="A132" s="39" t="n">
         <v>128</v>
       </c>
@@ -5786,7 +6670,7 @@
       <c r="L132" s="39" t="inlineStr"/>
       <c r="N132" s="39" t="inlineStr"/>
     </row>
-    <row r="133" ht="30" customHeight="1">
+    <row r="133" ht="46" customHeight="1">
       <c r="A133" s="39" t="n">
         <v>129</v>
       </c>
@@ -5830,7 +6714,7 @@
       <c r="L133" s="39" t="inlineStr"/>
       <c r="N133" s="39" t="inlineStr"/>
     </row>
-    <row r="134" ht="30" customHeight="1">
+    <row r="134" ht="46" customHeight="1">
       <c r="A134" s="39" t="n">
         <v>130</v>
       </c>
@@ -5870,11 +6754,23 @@
           <t>IQF mango 20x20 chunks (zebdya variety), 1x24t container</t>
         </is>
       </c>
-      <c r="J134" s="39" t="inlineStr"/>
-      <c r="L134" s="39" t="inlineStr"/>
-      <c r="N134" s="39" t="inlineStr"/>
-    </row>
-    <row r="135" ht="30" customHeight="1">
+      <c r="J134" s="39" t="inlineStr">
+        <is>
+          <t>One container - 24 tons</t>
+        </is>
+      </c>
+      <c r="L134" s="39" t="inlineStr">
+        <is>
+          <t>IQF mango 20x20 chunks, only Zebdya variety; asks price and lead time</t>
+        </is>
+      </c>
+      <c r="N134" s="39" t="inlineStr">
+        <is>
+          <t>Fresh Apple Turkey; Furkan Col, Manager; also requested online meeting; MAFI noted IQF production but no mango, start Q2 2026; Mobile +9053...</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="46" customHeight="1">
       <c r="A135" s="39" t="n">
         <v>131</v>
       </c>
@@ -5915,8 +6811,16 @@
         </is>
       </c>
       <c r="J135" s="39" t="inlineStr"/>
-      <c r="L135" s="39" t="inlineStr"/>
-      <c r="N135" s="39" t="inlineStr"/>
+      <c r="L135" s="39" t="inlineStr">
+        <is>
+          <t>Strawberry IQF; asks if MAFI can offer</t>
+        </is>
+      </c>
+      <c r="N135" s="39" t="inlineStr">
+        <is>
+          <t>Hellenic Juice Industry C. Dedes ASPIS S.A., Argos-Korinthos Greece; Mario Chronis, General Manager; T +302751028004, M +306951010008</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="410">

</xml_diff>